<commit_message>
Enhance: Integrate database management and improve Excel processing functionality
- Updated `excel_processor.py` to streamline database interactions by removing direct database parameter passing and utilizing a global database manager.
- Enhanced the `process_excel_file` function to handle database connections more efficiently, improving overall performance.
- Refactored the `show_excel_processor` function in `excel_processor_page.py` to enforce database loading requirements, ensuring smoother user experience.
- Improved the database selection process in `main.py` by implementing a more user-friendly interface for selecting and loading databases into memory.
- Added new utility functions in `common.py` for managing memory databases, enhancing the application's data handling capabilities.
</commit_message>
<xml_diff>
--- a/resources/Out_format.xlsx
+++ b/resources/Out_format.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\my_github\FlightCheckPy\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53C720C9-23EE-41E0-8162-CE60DC3D8BBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{950BD087-C01E-4909-BA88-E013711A771D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9084" yWindow="3456" windowWidth="16416" windowHeight="12156" xr2:uid="{D6DB75D4-A8CC-4A73-9AF5-6E324AED1BA5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{D6DB75D4-A8CC-4A73-9AF5-6E324AED1BA5}"/>
   </bookViews>
   <sheets>
     <sheet name="RECEIPT" sheetId="17" r:id="rId1"/>
@@ -32,6 +32,9 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -454,7 +457,7 @@
     <numFmt numFmtId="180" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="181" formatCode="00000"/>
   </numFmts>
-  <fonts count="41" x14ac:knownFonts="1">
+  <fonts count="42" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -699,6 +702,12 @@
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -1188,17 +1197,11 @@
     <xf numFmtId="26" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="180" fontId="9" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="26" fontId="28" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1225,14 +1228,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -1260,9 +1257,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="11" xfId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="177" fontId="7" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1278,50 +1272,56 @@
     <xf numFmtId="1" fontId="9" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="181" fontId="9" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="distributed"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="178" fontId="22" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="distributed"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="178" fontId="22" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1340,118 +1340,13 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="10" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="26" fontId="3" fillId="0" borderId="10" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1462,6 +1357,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1490,11 +1391,119 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="10" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="9" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="9" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="14">
@@ -1973,18 +1982,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D40067CD-9956-401A-A618-7A92843119E5}">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:L47"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.44140625" style="1" customWidth="1"/>
-    <col min="3" max="5" width="9.109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.109375" style="1" customWidth="1"/>
-    <col min="7" max="8" width="9.109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="10.88671875" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="1" width="11.625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5" style="1" customWidth="1"/>
+    <col min="3" max="5" width="9.125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.125" style="1" customWidth="1"/>
+    <col min="7" max="8" width="9.125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="10.875" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1997,37 +2006,37 @@
       <c r="J1" s="3"/>
       <c r="K1" s="3"/>
     </row>
-    <row r="2" spans="1:12" ht="22.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="C2" s="3"/>
-      <c r="D2" s="94" t="s">
+      <c r="D2" s="81" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="94"/>
-      <c r="F2" s="94"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="81"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="25"/>
     </row>
-    <row r="3" spans="1:12" ht="19.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="19.5" x14ac:dyDescent="0.25">
       <c r="A3" s="32"/>
       <c r="B3" s="32"/>
       <c r="C3" s="32"/>
-      <c r="D3" s="95" t="s">
+      <c r="D3" s="82" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="95"/>
-      <c r="F3" s="95"/>
-      <c r="G3" s="96" t="s">
+      <c r="E3" s="82"/>
+      <c r="F3" s="82"/>
+      <c r="G3" s="83" t="s">
         <v>46</v>
       </c>
-      <c r="H3" s="96"/>
-      <c r="I3" s="96"/>
+      <c r="H3" s="83"/>
+      <c r="I3" s="83"/>
       <c r="J3" s="35"/>
       <c r="K3" s="35"/>
       <c r="L3" s="34"/>
     </row>
-    <row r="4" spans="1:12" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" s="24"/>
       <c r="B4" s="24"/>
       <c r="C4" s="24"/>
@@ -2040,201 +2049,201 @@
       <c r="J4" s="24"/>
       <c r="K4" s="24"/>
     </row>
-    <row r="5" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="89" t="s">
+    <row r="5" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="84" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="89"/>
-      <c r="C5" s="86">
+      <c r="B5" s="84"/>
+      <c r="C5" s="85">
         <f>SUM!C13</f>
         <v>0</v>
       </c>
-      <c r="D5" s="86"/>
-      <c r="E5" s="86"/>
-      <c r="F5" s="97" t="s">
+      <c r="D5" s="85"/>
+      <c r="E5" s="85"/>
+      <c r="F5" s="87" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="99">
+      <c r="G5" s="89">
         <f>SUM!G11</f>
         <v>0</v>
       </c>
-      <c r="H5" s="99"/>
-      <c r="I5" s="99"/>
+      <c r="H5" s="89"/>
+      <c r="I5" s="89"/>
       <c r="J5" s="33"/>
       <c r="K5" s="33"/>
     </row>
-    <row r="6" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="90" t="s">
+    <row r="6" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="91" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="90"/>
-      <c r="C6" s="87"/>
-      <c r="D6" s="87"/>
-      <c r="E6" s="87"/>
-      <c r="F6" s="98"/>
-      <c r="G6" s="100"/>
-      <c r="H6" s="100"/>
-      <c r="I6" s="100"/>
+      <c r="B6" s="91"/>
+      <c r="C6" s="86"/>
+      <c r="D6" s="86"/>
+      <c r="E6" s="86"/>
+      <c r="F6" s="88"/>
+      <c r="G6" s="90"/>
+      <c r="H6" s="90"/>
+      <c r="I6" s="90"/>
       <c r="J6" s="33"/>
       <c r="K6" s="33"/>
     </row>
-    <row r="8" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="93" t="s">
+    <row r="8" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="92" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="93"/>
-      <c r="C8" s="157"/>
-      <c r="D8" s="157"/>
-      <c r="E8" s="157"/>
-      <c r="F8" s="157"/>
-      <c r="G8" s="157"/>
-      <c r="H8" s="157"/>
-      <c r="I8" s="157"/>
-    </row>
-    <row r="9" spans="1:12" ht="49.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="93"/>
-      <c r="B9" s="93"/>
-      <c r="C9" s="158"/>
-      <c r="D9" s="158"/>
-      <c r="E9" s="158"/>
-      <c r="F9" s="158"/>
-      <c r="G9" s="158"/>
-      <c r="H9" s="158"/>
-      <c r="I9" s="158"/>
-    </row>
-    <row r="11" spans="1:12" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A11" s="89" t="s">
+      <c r="B8" s="92"/>
+      <c r="C8" s="93"/>
+      <c r="D8" s="93"/>
+      <c r="E8" s="93"/>
+      <c r="F8" s="93"/>
+      <c r="G8" s="93"/>
+      <c r="H8" s="93"/>
+      <c r="I8" s="93"/>
+    </row>
+    <row r="9" spans="1:12" ht="49.7" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="92"/>
+      <c r="B9" s="92"/>
+      <c r="C9" s="94"/>
+      <c r="D9" s="94"/>
+      <c r="E9" s="94"/>
+      <c r="F9" s="94"/>
+      <c r="G9" s="94"/>
+      <c r="H9" s="94"/>
+      <c r="I9" s="94"/>
+    </row>
+    <row r="11" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A11" s="84" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="89"/>
-      <c r="C11" s="86" t="s">
+      <c r="B11" s="84"/>
+      <c r="C11" s="85" t="s">
         <v>50</v>
       </c>
-      <c r="D11" s="86"/>
-      <c r="E11" s="86"/>
+      <c r="D11" s="85"/>
+      <c r="E11" s="85"/>
       <c r="F11" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="G11" s="88">
+      <c r="G11" s="95">
         <f>SUM!C14</f>
         <v>0</v>
       </c>
-      <c r="H11" s="86"/>
-      <c r="I11" s="86"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="90" t="s">
+      <c r="H11" s="85"/>
+      <c r="I11" s="85"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12" s="91" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="90"/>
-      <c r="C12" s="87"/>
-      <c r="D12" s="87"/>
-      <c r="E12" s="87"/>
+      <c r="B12" s="91"/>
+      <c r="C12" s="86"/>
+      <c r="D12" s="86"/>
+      <c r="E12" s="86"/>
       <c r="F12" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="G12" s="87"/>
-      <c r="H12" s="87"/>
-      <c r="I12" s="87"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="89" t="s">
+      <c r="G12" s="86"/>
+      <c r="H12" s="86"/>
+      <c r="I12" s="86"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" s="84" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="89"/>
-      <c r="C14" s="86" t="s">
+      <c r="B14" s="84"/>
+      <c r="C14" s="85" t="s">
         <v>78</v>
       </c>
-      <c r="D14" s="86"/>
-      <c r="E14" s="86"/>
-      <c r="F14" s="86"/>
-      <c r="G14" s="86"/>
-      <c r="H14" s="86"/>
-      <c r="I14" s="86"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="90" t="s">
+      <c r="D14" s="85"/>
+      <c r="E14" s="85"/>
+      <c r="F14" s="85"/>
+      <c r="G14" s="85"/>
+      <c r="H14" s="85"/>
+      <c r="I14" s="85"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A15" s="91" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="90"/>
-      <c r="C15" s="87"/>
-      <c r="D15" s="87"/>
-      <c r="E15" s="87"/>
-      <c r="F15" s="87"/>
-      <c r="G15" s="87"/>
-      <c r="H15" s="87"/>
-      <c r="I15" s="87"/>
-    </row>
-    <row r="17" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="91"/>
+      <c r="C15" s="86"/>
+      <c r="D15" s="86"/>
+      <c r="E15" s="86"/>
+      <c r="F15" s="86"/>
+      <c r="G15" s="86"/>
+      <c r="H15" s="86"/>
+      <c r="I15" s="86"/>
+    </row>
+    <row r="17" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="B17" s="86" t="s">
+      <c r="B17" s="85" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="86"/>
-      <c r="D17" s="86"/>
-      <c r="E17" s="86"/>
+      <c r="C17" s="85"/>
+      <c r="D17" s="85"/>
+      <c r="E17" s="85"/>
       <c r="F17" s="31" t="s">
         <v>58</v>
       </c>
       <c r="G17" s="31"/>
-      <c r="H17" s="86" t="s">
+      <c r="H17" s="85" t="s">
         <v>59</v>
       </c>
-      <c r="I17" s="86"/>
-    </row>
-    <row r="18" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I17" s="85"/>
+    </row>
+    <row r="18" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="B18" s="87"/>
-      <c r="C18" s="87"/>
-      <c r="D18" s="87"/>
-      <c r="E18" s="87"/>
-      <c r="F18" s="91" t="s">
+      <c r="B18" s="86"/>
+      <c r="C18" s="86"/>
+      <c r="D18" s="86"/>
+      <c r="E18" s="86"/>
+      <c r="F18" s="96" t="s">
         <v>61</v>
       </c>
-      <c r="G18" s="92"/>
-      <c r="H18" s="87"/>
-      <c r="I18" s="87"/>
-    </row>
-    <row r="20" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G18" s="97"/>
+      <c r="H18" s="86"/>
+      <c r="I18" s="86"/>
+    </row>
+    <row r="20" spans="1:9" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="86" t="s">
+      <c r="B20" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="86"/>
-      <c r="D20" s="86"/>
-      <c r="E20" s="86"/>
+      <c r="C20" s="85"/>
+      <c r="D20" s="85"/>
+      <c r="E20" s="85"/>
       <c r="F20" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="G20" s="88">
+      <c r="G20" s="95">
         <f>SUM!C14</f>
         <v>0</v>
       </c>
-      <c r="H20" s="86"/>
-      <c r="I20" s="86"/>
-    </row>
-    <row r="21" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H20" s="85"/>
+      <c r="I20" s="85"/>
+    </row>
+    <row r="21" spans="1:9" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="B21" s="87"/>
-      <c r="C21" s="87"/>
-      <c r="D21" s="87"/>
-      <c r="E21" s="87"/>
+      <c r="B21" s="86"/>
+      <c r="C21" s="86"/>
+      <c r="D21" s="86"/>
+      <c r="E21" s="86"/>
       <c r="F21" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="G21" s="87"/>
-      <c r="H21" s="87"/>
-      <c r="I21" s="87"/>
-    </row>
-    <row r="22" spans="1:9" ht="19.8" x14ac:dyDescent="0.35">
+      <c r="G21" s="86"/>
+      <c r="H21" s="86"/>
+      <c r="I21" s="86"/>
+    </row>
+    <row r="22" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A22" s="27"/>
       <c r="B22" s="28"/>
       <c r="C22" s="28"/>
@@ -2245,21 +2254,35 @@
       <c r="H22" s="28"/>
       <c r="I22" s="28"/>
     </row>
-    <row r="23" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="46.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="14.4" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="31" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="34" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="35" ht="46.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="37" ht="14.45" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="38" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="40" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="43" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B20:E21"/>
+    <mergeCell ref="G20:I21"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:I15"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="B17:E18"/>
+    <mergeCell ref="H17:I18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="A8:B9"/>
+    <mergeCell ref="C8:I9"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:E12"/>
+    <mergeCell ref="G11:I12"/>
+    <mergeCell ref="A12:B12"/>
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="D3:F3"/>
     <mergeCell ref="G3:I3"/>
@@ -2268,20 +2291,6 @@
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="G5:I6"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A8:B9"/>
-    <mergeCell ref="C8:I9"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:E12"/>
-    <mergeCell ref="G11:I12"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="B20:E21"/>
-    <mergeCell ref="G20:I21"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:I15"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="B17:E18"/>
-    <mergeCell ref="H17:I18"/>
-    <mergeCell ref="F18:G18"/>
   </mergeCells>
   <phoneticPr fontId="40" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2298,26 +2307,26 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N26"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.44140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="3.375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5" style="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.6640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="15.44140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="16.44140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="16.109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="11.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.44140625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="9.109375" style="1"/>
+    <col min="7" max="7" width="15.625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5" style="1" customWidth="1"/>
+    <col min="10" max="10" width="16.625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="16.125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5" style="1" customWidth="1"/>
+    <col min="14" max="14" width="10.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="15" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2330,7 +2339,7 @@
       <c r="J1" s="36"/>
       <c r="K1" s="37"/>
     </row>
-    <row r="2" spans="1:14" ht="19.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="19.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -2342,25 +2351,25 @@
       <c r="J2" s="3"/>
       <c r="K2" s="25"/>
     </row>
-    <row r="3" spans="1:14" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="104" t="s">
+    <row r="3" spans="1:14" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="101" t="s">
         <v>74</v>
       </c>
-      <c r="B3" s="104"/>
-      <c r="C3" s="104"/>
-      <c r="D3" s="104"/>
-      <c r="E3" s="104"/>
-      <c r="F3" s="104"/>
-      <c r="G3" s="104"/>
-      <c r="H3" s="104"/>
-      <c r="I3" s="104"/>
-      <c r="J3" s="104"/>
-      <c r="K3" s="104"/>
+      <c r="B3" s="101"/>
+      <c r="C3" s="101"/>
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="101"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="101"/>
+      <c r="J3" s="101"/>
+      <c r="K3" s="101"/>
       <c r="L3" s="23"/>
       <c r="M3" s="23"/>
       <c r="N3" s="23"/>
     </row>
-    <row r="4" spans="1:14" ht="22.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A4" s="24"/>
       <c r="B4" s="24"/>
       <c r="C4" s="24"/>
@@ -2370,17 +2379,17 @@
       <c r="G4" s="24"/>
       <c r="H4" s="24"/>
       <c r="I4" s="24"/>
-      <c r="J4" s="82" t="s">
+      <c r="J4" s="77" t="s">
         <v>80</v>
       </c>
-      <c r="K4" s="81">
+      <c r="K4" s="76">
         <v>984</v>
       </c>
       <c r="L4" s="23"/>
       <c r="M4" s="23"/>
       <c r="N4" s="23"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -2393,7 +2402,7 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:14" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="22" t="s">
         <v>18</v>
       </c>
@@ -2410,66 +2419,66 @@
         <v>00-Jan-1900</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="21"/>
-      <c r="B7" s="107" t="s">
+      <c r="B7" s="104" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="101" t="s">
+      <c r="C7" s="98" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="101" t="s">
+      <c r="D7" s="98" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="101" t="s">
+      <c r="E7" s="98" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="101" t="s">
+      <c r="F7" s="98" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="101" t="s">
+      <c r="G7" s="98" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="105" t="s">
+      <c r="H7" s="102" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="106"/>
-      <c r="J7" s="101" t="s">
+      <c r="I7" s="103"/>
+      <c r="J7" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="K7" s="101" t="s">
+      <c r="K7" s="98" t="s">
         <v>9</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="8"/>
     </row>
-    <row r="8" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="21"/>
-      <c r="B8" s="107"/>
-      <c r="C8" s="101"/>
-      <c r="D8" s="101"/>
-      <c r="E8" s="101"/>
-      <c r="F8" s="101"/>
-      <c r="G8" s="101"/>
+      <c r="B8" s="104"/>
+      <c r="C8" s="98"/>
+      <c r="D8" s="98"/>
+      <c r="E8" s="98"/>
+      <c r="F8" s="98"/>
+      <c r="G8" s="98"/>
       <c r="H8" s="20" t="s">
         <v>8</v>
       </c>
       <c r="I8" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="J8" s="101"/>
-      <c r="K8" s="101"/>
+      <c r="J8" s="98"/>
+      <c r="K8" s="98"/>
       <c r="L8" s="2"/>
       <c r="M8" s="8"/>
     </row>
-    <row r="9" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="13">
         <v>1</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="79">
+      <c r="C9" s="74">
         <f>EMD!B29</f>
         <v>0</v>
       </c>
@@ -2502,7 +2511,7 @@
       <c r="L9" s="2"/>
       <c r="M9" s="15"/>
     </row>
-    <row r="10" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="13">
         <v>2</v>
       </c>
@@ -2520,7 +2529,7 @@
       <c r="M10" s="15"/>
       <c r="N10" s="8"/>
     </row>
-    <row r="11" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="13">
         <v>6</v>
       </c>
@@ -2563,7 +2572,7 @@
       <c r="L11" s="2"/>
       <c r="M11" s="8"/>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="D12" s="3"/>
@@ -2575,7 +2584,7 @@
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>6</v>
       </c>
@@ -2590,11 +2599,11 @@
       <c r="J13" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="K13" s="80" t="s">
+      <c r="K13" s="75" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>4</v>
       </c>
@@ -2616,7 +2625,7 @@
         <v>00-Jan-1900</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="6"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -2629,7 +2638,7 @@
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="D16" s="3"/>
@@ -2641,7 +2650,7 @@
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -2654,7 +2663,7 @@
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -2667,7 +2676,7 @@
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="5"/>
@@ -2680,7 +2689,7 @@
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="5"/>
@@ -2693,27 +2702,27 @@
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
     </row>
-    <row r="21" spans="1:11" ht="15" x14ac:dyDescent="0.25">
-      <c r="C21" s="102"/>
-      <c r="D21" s="103"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+      <c r="C21" s="99"/>
+      <c r="D21" s="100"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
     </row>
@@ -2748,593 +2757,593 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="18.5546875" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" customWidth="1"/>
-    <col min="3" max="3" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" customWidth="1"/>
-    <col min="6" max="6" width="7.6640625" customWidth="1"/>
-    <col min="7" max="7" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.5546875" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="18.5" customWidth="1"/>
+    <col min="2" max="2" width="16.125" customWidth="1"/>
+    <col min="3" max="3" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5" customWidth="1"/>
+    <col min="5" max="5" width="13.625" customWidth="1"/>
+    <col min="6" max="6" width="7.625" customWidth="1"/>
+    <col min="7" max="7" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5" customWidth="1"/>
+    <col min="9" max="9" width="11.625" customWidth="1"/>
     <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="11" max="11" width="10.6640625" customWidth="1"/>
-    <col min="12" max="12" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.109375" customWidth="1"/>
+    <col min="11" max="11" width="10.625" customWidth="1"/>
+    <col min="12" max="12" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.125" customWidth="1"/>
     <col min="14" max="14" width="11" customWidth="1"/>
-    <col min="15" max="15" width="14.5546875" customWidth="1"/>
-    <col min="16" max="16" width="9.5546875" customWidth="1"/>
-    <col min="17" max="17" width="13.6640625" customWidth="1"/>
-    <col min="18" max="18" width="12.33203125" customWidth="1"/>
+    <col min="15" max="15" width="14.5" customWidth="1"/>
+    <col min="16" max="16" width="9.5" customWidth="1"/>
+    <col min="17" max="17" width="13.625" customWidth="1"/>
+    <col min="18" max="18" width="12.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="108" t="s">
+    <row r="1" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="121" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="108"/>
-      <c r="I1" s="108"/>
-      <c r="J1" s="108"/>
-      <c r="K1" s="108"/>
-      <c r="L1" s="108"/>
-      <c r="M1" s="108"/>
-      <c r="N1" s="108"/>
-      <c r="O1" s="108"/>
-      <c r="P1" s="108"/>
-      <c r="Q1" s="72"/>
-      <c r="R1" s="72"/>
-      <c r="S1" s="72"/>
-    </row>
-    <row r="2" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="109" t="s">
+      <c r="B1" s="121"/>
+      <c r="C1" s="121"/>
+      <c r="D1" s="121"/>
+      <c r="E1" s="121"/>
+      <c r="F1" s="121"/>
+      <c r="G1" s="121"/>
+      <c r="H1" s="121"/>
+      <c r="I1" s="121"/>
+      <c r="J1" s="121"/>
+      <c r="K1" s="121"/>
+      <c r="L1" s="121"/>
+      <c r="M1" s="121"/>
+      <c r="N1" s="121"/>
+      <c r="O1" s="121"/>
+      <c r="P1" s="121"/>
+      <c r="Q1" s="68"/>
+      <c r="R1" s="68"/>
+      <c r="S1" s="68"/>
+    </row>
+    <row r="2" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="122" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="109"/>
-      <c r="C2" s="109"/>
-      <c r="D2" s="109"/>
-      <c r="E2" s="109"/>
-      <c r="F2" s="109"/>
-      <c r="G2" s="109"/>
-      <c r="H2" s="109"/>
-      <c r="I2" s="109"/>
-      <c r="J2" s="109"/>
-      <c r="K2" s="109"/>
-      <c r="L2" s="109"/>
-      <c r="M2" s="109"/>
-      <c r="N2" s="109"/>
-      <c r="O2" s="109"/>
-      <c r="P2" s="109"/>
-      <c r="Q2" s="73"/>
-      <c r="R2" s="73"/>
-      <c r="S2" s="73"/>
-    </row>
-    <row r="3" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="122"/>
+      <c r="C2" s="122"/>
+      <c r="D2" s="122"/>
+      <c r="E2" s="122"/>
+      <c r="F2" s="122"/>
+      <c r="G2" s="122"/>
+      <c r="H2" s="122"/>
+      <c r="I2" s="122"/>
+      <c r="J2" s="122"/>
+      <c r="K2" s="122"/>
+      <c r="L2" s="122"/>
+      <c r="M2" s="122"/>
+      <c r="N2" s="122"/>
+      <c r="O2" s="122"/>
+      <c r="P2" s="122"/>
+      <c r="Q2" s="69"/>
+      <c r="R2" s="69"/>
+      <c r="S2" s="69"/>
+    </row>
+    <row r="3" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="44" t="s">
         <v>77</v>
       </c>
       <c r="B3" s="44"/>
       <c r="C3" s="44"/>
-      <c r="E3" s="143" t="str">
+      <c r="E3" s="106" t="str">
         <f>"报告期间：" &amp; N3 &amp; "至" &amp; N3</f>
         <v>报告期间：1900年1月0日至1900年1月0日</v>
       </c>
-      <c r="F3" s="143"/>
-      <c r="G3" s="143"/>
-      <c r="H3" s="143"/>
-      <c r="I3" s="143"/>
-      <c r="J3" s="143" t="s">
+      <c r="F3" s="106"/>
+      <c r="G3" s="106"/>
+      <c r="H3" s="106"/>
+      <c r="I3" s="106"/>
+      <c r="J3" s="106" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="143"/>
+      <c r="K3" s="106"/>
       <c r="L3" s="43"/>
-      <c r="M3" s="70"/>
-      <c r="N3" s="70" t="str">
+      <c r="M3" s="66"/>
+      <c r="N3" s="66" t="str">
         <f>YEAR(SUM!C14) &amp; "年" &amp; MONTH(SUM!C14) &amp; "月" &amp; DAY(SUM!C14)&amp;"日"</f>
         <v>1900年1月0日</v>
       </c>
       <c r="O3" s="43"/>
       <c r="P3" s="43"/>
       <c r="Q3" s="45"/>
-      <c r="R3" s="53"/>
+      <c r="R3" s="51"/>
       <c r="S3" s="45"/>
     </row>
-    <row r="4" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="145" t="s">
+    <row r="4" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="107" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="145"/>
-      <c r="C4" s="145"/>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74"/>
-      <c r="F4" s="75"/>
-      <c r="G4" s="76"/>
-      <c r="H4" s="146"/>
-      <c r="I4" s="146"/>
-      <c r="J4" s="71" t="s">
+      <c r="B4" s="107"/>
+      <c r="C4" s="107"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="70"/>
+      <c r="F4" s="71"/>
+      <c r="G4" s="72"/>
+      <c r="H4" s="108"/>
+      <c r="I4" s="108"/>
+      <c r="J4" s="67" t="s">
         <v>76</v>
       </c>
-      <c r="K4" s="71"/>
-      <c r="L4" s="71"/>
-      <c r="M4" s="71" t="str">
+      <c r="K4" s="67"/>
+      <c r="L4" s="67"/>
+      <c r="M4" s="67" t="str">
         <f>"REPORT NO: " &amp; TEXT(SUM!C14,"YYMMDD") &amp; "CA" &amp; SUM!K4 &amp;"EMD"</f>
         <v>REPORT NO: 000100CA984EMD</v>
       </c>
-      <c r="N4" s="71"/>
-      <c r="O4" s="71"/>
-      <c r="P4" s="71"/>
-    </row>
-    <row r="5" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="155" t="s">
+      <c r="N4" s="67"/>
+      <c r="O4" s="67"/>
+      <c r="P4" s="67"/>
+    </row>
+    <row r="5" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="119" t="s">
         <v>70</v>
       </c>
-      <c r="B5" s="153" t="s">
+      <c r="B5" s="117" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="151" t="s">
+      <c r="C5" s="115" t="s">
         <v>72</v>
       </c>
-      <c r="D5" s="141" t="s">
+      <c r="D5" s="111" t="s">
         <v>73</v>
       </c>
-      <c r="E5" s="147" t="s">
+      <c r="E5" s="109" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="141" t="s">
+      <c r="F5" s="111" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="147" t="s">
+      <c r="G5" s="109" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="147" t="s">
+      <c r="H5" s="109" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="147" t="s">
+      <c r="I5" s="109" t="s">
         <v>28</v>
       </c>
-      <c r="J5" s="147" t="s">
+      <c r="J5" s="109" t="s">
         <v>29</v>
       </c>
-      <c r="K5" s="141" t="s">
+      <c r="K5" s="111" t="s">
         <v>24</v>
       </c>
-      <c r="L5" s="149" t="s">
+      <c r="L5" s="113" t="s">
         <v>41</v>
       </c>
-      <c r="M5" s="149" t="s">
+      <c r="M5" s="113" t="s">
         <v>42</v>
       </c>
-      <c r="N5" s="149"/>
-      <c r="O5" s="59" t="s">
+      <c r="N5" s="113"/>
+      <c r="O5" s="57" t="s">
         <v>66</v>
       </c>
-      <c r="P5" s="60" t="s">
+      <c r="P5" s="58" t="s">
         <v>67</v>
       </c>
-      <c r="Q5" s="144"/>
-      <c r="R5" s="144"/>
-    </row>
-    <row r="6" spans="1:19" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="156"/>
-      <c r="B6" s="154"/>
-      <c r="C6" s="152"/>
-      <c r="D6" s="142"/>
-      <c r="E6" s="148"/>
-      <c r="F6" s="142"/>
-      <c r="G6" s="148"/>
-      <c r="H6" s="148"/>
-      <c r="I6" s="148"/>
-      <c r="J6" s="148"/>
-      <c r="K6" s="142"/>
-      <c r="L6" s="150"/>
-      <c r="M6" s="55" t="s">
+      <c r="Q5" s="105"/>
+      <c r="R5" s="105"/>
+    </row>
+    <row r="6" spans="1:19" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="120"/>
+      <c r="B6" s="118"/>
+      <c r="C6" s="116"/>
+      <c r="D6" s="112"/>
+      <c r="E6" s="110"/>
+      <c r="F6" s="112"/>
+      <c r="G6" s="110"/>
+      <c r="H6" s="110"/>
+      <c r="I6" s="110"/>
+      <c r="J6" s="110"/>
+      <c r="K6" s="112"/>
+      <c r="L6" s="114"/>
+      <c r="M6" s="53" t="s">
         <v>43</v>
       </c>
-      <c r="N6" s="55" t="s">
+      <c r="N6" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="O6" s="54" t="s">
+      <c r="O6" s="52" t="s">
         <v>68</v>
       </c>
-      <c r="P6" s="61" t="s">
+      <c r="P6" s="59" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A7" s="156"/>
-      <c r="B7" s="154"/>
-      <c r="C7" s="152"/>
-      <c r="D7" s="142"/>
-      <c r="E7" s="148"/>
-      <c r="F7" s="142"/>
-      <c r="G7" s="148"/>
-      <c r="H7" s="148"/>
-      <c r="I7" s="148"/>
-      <c r="J7" s="148"/>
-      <c r="K7" s="142"/>
-      <c r="L7" s="56"/>
-      <c r="M7" s="56"/>
-      <c r="N7" s="56"/>
-      <c r="O7" s="56">
+    <row r="7" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A7" s="120"/>
+      <c r="B7" s="118"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="112"/>
+      <c r="E7" s="110"/>
+      <c r="F7" s="112"/>
+      <c r="G7" s="110"/>
+      <c r="H7" s="110"/>
+      <c r="I7" s="110"/>
+      <c r="J7" s="110"/>
+      <c r="K7" s="112"/>
+      <c r="L7" s="54"/>
+      <c r="M7" s="54"/>
+      <c r="N7" s="54"/>
+      <c r="O7" s="54">
         <v>9</v>
       </c>
-      <c r="P7" s="61">
+      <c r="P7" s="59">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A8" s="83"/>
-      <c r="B8" s="84"/>
+    <row r="8" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A8" s="78"/>
+      <c r="B8" s="79"/>
       <c r="C8" s="42"/>
       <c r="D8" s="42"/>
       <c r="E8" s="42"/>
       <c r="F8" s="42"/>
-      <c r="G8" s="57"/>
-      <c r="H8" s="77"/>
-      <c r="I8" s="77"/>
+      <c r="G8" s="55"/>
+      <c r="H8" s="73"/>
+      <c r="I8" s="73"/>
       <c r="J8" s="42"/>
-      <c r="K8" s="52"/>
-      <c r="L8" s="52"/>
-      <c r="M8" s="52"/>
-      <c r="N8" s="52"/>
-      <c r="O8" s="78"/>
-      <c r="P8" s="63"/>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A9" s="83"/>
-      <c r="B9" s="85"/>
+      <c r="K8" s="50"/>
+      <c r="L8" s="50"/>
+      <c r="M8" s="50"/>
+      <c r="N8" s="50"/>
+      <c r="O8" s="154"/>
+      <c r="P8" s="155"/>
+    </row>
+    <row r="9" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A9" s="78"/>
+      <c r="B9" s="80"/>
       <c r="C9" s="42"/>
       <c r="D9" s="42"/>
       <c r="E9" s="42"/>
       <c r="F9" s="42"/>
-      <c r="G9" s="57"/>
-      <c r="H9" s="77"/>
-      <c r="I9" s="77"/>
+      <c r="G9" s="55"/>
+      <c r="H9" s="73"/>
+      <c r="I9" s="73"/>
       <c r="J9" s="42"/>
-      <c r="K9" s="52"/>
-      <c r="L9" s="52"/>
-      <c r="M9" s="52"/>
-      <c r="N9" s="52"/>
-      <c r="O9" s="46"/>
-      <c r="P9" s="63"/>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A10" s="83"/>
-      <c r="B10" s="85"/>
+      <c r="K9" s="50"/>
+      <c r="L9" s="50"/>
+      <c r="M9" s="50"/>
+      <c r="N9" s="50"/>
+      <c r="O9" s="156"/>
+      <c r="P9" s="155"/>
+    </row>
+    <row r="10" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A10" s="78"/>
+      <c r="B10" s="80"/>
       <c r="C10" s="42"/>
       <c r="D10" s="42"/>
       <c r="E10" s="42"/>
       <c r="F10" s="42"/>
-      <c r="G10" s="57"/>
-      <c r="H10" s="77"/>
-      <c r="I10" s="77"/>
+      <c r="G10" s="55"/>
+      <c r="H10" s="73"/>
+      <c r="I10" s="73"/>
       <c r="J10" s="42"/>
-      <c r="K10" s="52"/>
-      <c r="L10" s="52"/>
-      <c r="M10" s="52"/>
-      <c r="N10" s="52"/>
-      <c r="O10" s="46"/>
-      <c r="P10" s="63"/>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A11" s="83"/>
-      <c r="B11" s="85"/>
+      <c r="K10" s="50"/>
+      <c r="L10" s="50"/>
+      <c r="M10" s="50"/>
+      <c r="N10" s="50"/>
+      <c r="O10" s="156"/>
+      <c r="P10" s="155"/>
+    </row>
+    <row r="11" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A11" s="78"/>
+      <c r="B11" s="80"/>
       <c r="C11" s="42"/>
       <c r="D11" s="42"/>
       <c r="E11" s="42"/>
       <c r="F11" s="42"/>
-      <c r="G11" s="57"/>
-      <c r="H11" s="77"/>
-      <c r="I11" s="77"/>
+      <c r="G11" s="55"/>
+      <c r="H11" s="73"/>
+      <c r="I11" s="73"/>
       <c r="J11" s="42"/>
-      <c r="K11" s="52"/>
-      <c r="L11" s="52"/>
-      <c r="M11" s="52"/>
-      <c r="N11" s="52"/>
-      <c r="O11" s="46"/>
-      <c r="P11" s="63"/>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A12" s="83"/>
-      <c r="B12" s="85"/>
+      <c r="K11" s="50"/>
+      <c r="L11" s="50"/>
+      <c r="M11" s="50"/>
+      <c r="N11" s="50"/>
+      <c r="O11" s="156"/>
+      <c r="P11" s="155"/>
+    </row>
+    <row r="12" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A12" s="78"/>
+      <c r="B12" s="80"/>
       <c r="C12" s="42"/>
       <c r="D12" s="42"/>
       <c r="E12" s="42"/>
       <c r="F12" s="42"/>
-      <c r="G12" s="57"/>
-      <c r="H12" s="77"/>
-      <c r="I12" s="77"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="73"/>
+      <c r="I12" s="73"/>
       <c r="J12" s="42"/>
-      <c r="K12" s="52"/>
-      <c r="L12" s="52"/>
-      <c r="M12" s="52"/>
-      <c r="N12" s="52"/>
-      <c r="O12" s="46"/>
-      <c r="P12" s="63"/>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A13" s="83"/>
-      <c r="B13" s="84"/>
+      <c r="K12" s="50"/>
+      <c r="L12" s="50"/>
+      <c r="M12" s="50"/>
+      <c r="N12" s="50"/>
+      <c r="O12" s="156"/>
+      <c r="P12" s="155"/>
+    </row>
+    <row r="13" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A13" s="78"/>
+      <c r="B13" s="79"/>
       <c r="C13" s="42"/>
       <c r="D13" s="42"/>
       <c r="E13" s="42"/>
       <c r="F13" s="42"/>
-      <c r="G13" s="57"/>
-      <c r="H13" s="77"/>
-      <c r="I13" s="77"/>
+      <c r="G13" s="55"/>
+      <c r="H13" s="73"/>
+      <c r="I13" s="73"/>
       <c r="J13" s="42"/>
-      <c r="K13" s="52"/>
-      <c r="L13" s="52"/>
-      <c r="M13" s="52"/>
-      <c r="N13" s="52"/>
-      <c r="O13" s="78"/>
-      <c r="P13" s="63"/>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A14" s="83"/>
-      <c r="B14" s="85"/>
+      <c r="K13" s="50"/>
+      <c r="L13" s="50"/>
+      <c r="M13" s="50"/>
+      <c r="N13" s="50"/>
+      <c r="O13" s="154"/>
+      <c r="P13" s="155"/>
+    </row>
+    <row r="14" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A14" s="78"/>
+      <c r="B14" s="80"/>
       <c r="C14" s="42"/>
       <c r="D14" s="42"/>
       <c r="E14" s="42"/>
       <c r="F14" s="42"/>
-      <c r="G14" s="57"/>
-      <c r="H14" s="77"/>
-      <c r="I14" s="77"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="73"/>
+      <c r="I14" s="73"/>
       <c r="J14" s="42"/>
-      <c r="K14" s="52"/>
-      <c r="L14" s="52"/>
-      <c r="M14" s="52"/>
-      <c r="N14" s="52"/>
-      <c r="O14" s="46"/>
-      <c r="P14" s="63"/>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A15" s="83"/>
-      <c r="B15" s="85"/>
+      <c r="K14" s="50"/>
+      <c r="L14" s="50"/>
+      <c r="M14" s="50"/>
+      <c r="N14" s="50"/>
+      <c r="O14" s="156"/>
+      <c r="P14" s="155"/>
+    </row>
+    <row r="15" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A15" s="78"/>
+      <c r="B15" s="80"/>
       <c r="C15" s="42"/>
       <c r="D15" s="42"/>
       <c r="E15" s="42"/>
       <c r="F15" s="42"/>
-      <c r="G15" s="57"/>
-      <c r="H15" s="77"/>
-      <c r="I15" s="77"/>
+      <c r="G15" s="55"/>
+      <c r="H15" s="73"/>
+      <c r="I15" s="73"/>
       <c r="J15" s="42"/>
-      <c r="K15" s="52"/>
-      <c r="L15" s="52"/>
-      <c r="M15" s="52"/>
-      <c r="N15" s="52"/>
-      <c r="O15" s="46"/>
-      <c r="P15" s="63"/>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A16" s="83"/>
-      <c r="B16" s="85"/>
+      <c r="K15" s="50"/>
+      <c r="L15" s="50"/>
+      <c r="M15" s="50"/>
+      <c r="N15" s="50"/>
+      <c r="O15" s="156"/>
+      <c r="P15" s="155"/>
+    </row>
+    <row r="16" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A16" s="78"/>
+      <c r="B16" s="80"/>
       <c r="C16" s="42"/>
       <c r="D16" s="42"/>
       <c r="E16" s="42"/>
       <c r="F16" s="42"/>
-      <c r="G16" s="57"/>
-      <c r="H16" s="77"/>
-      <c r="I16" s="77"/>
+      <c r="G16" s="55"/>
+      <c r="H16" s="73"/>
+      <c r="I16" s="73"/>
       <c r="J16" s="42"/>
-      <c r="K16" s="52"/>
-      <c r="L16" s="52"/>
-      <c r="M16" s="52"/>
-      <c r="N16" s="52"/>
-      <c r="O16" s="46"/>
-      <c r="P16" s="63"/>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A17" s="83"/>
-      <c r="B17" s="85"/>
+      <c r="K16" s="50"/>
+      <c r="L16" s="50"/>
+      <c r="M16" s="50"/>
+      <c r="N16" s="50"/>
+      <c r="O16" s="156"/>
+      <c r="P16" s="155"/>
+    </row>
+    <row r="17" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A17" s="78"/>
+      <c r="B17" s="80"/>
       <c r="C17" s="42"/>
       <c r="D17" s="42"/>
       <c r="E17" s="42"/>
       <c r="F17" s="42"/>
-      <c r="G17" s="57"/>
-      <c r="H17" s="77"/>
-      <c r="I17" s="77"/>
+      <c r="G17" s="55"/>
+      <c r="H17" s="73"/>
+      <c r="I17" s="73"/>
       <c r="J17" s="42"/>
-      <c r="K17" s="52"/>
-      <c r="L17" s="52"/>
-      <c r="M17" s="52"/>
-      <c r="N17" s="52"/>
-      <c r="O17" s="46"/>
-      <c r="P17" s="63"/>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A18" s="83"/>
-      <c r="B18" s="85"/>
+      <c r="K17" s="50"/>
+      <c r="L17" s="50"/>
+      <c r="M17" s="50"/>
+      <c r="N17" s="50"/>
+      <c r="O17" s="156"/>
+      <c r="P17" s="155"/>
+    </row>
+    <row r="18" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A18" s="78"/>
+      <c r="B18" s="80"/>
       <c r="C18" s="42"/>
       <c r="D18" s="42"/>
       <c r="E18" s="42"/>
       <c r="F18" s="42"/>
-      <c r="G18" s="57"/>
-      <c r="H18" s="77"/>
-      <c r="I18" s="77"/>
+      <c r="G18" s="55"/>
+      <c r="H18" s="73"/>
+      <c r="I18" s="73"/>
       <c r="J18" s="42"/>
-      <c r="K18" s="52"/>
-      <c r="L18" s="52"/>
-      <c r="M18" s="52"/>
-      <c r="N18" s="52"/>
-      <c r="O18" s="46"/>
-      <c r="P18" s="63"/>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A19" s="83"/>
-      <c r="B19" s="85"/>
+      <c r="K18" s="50"/>
+      <c r="L18" s="50"/>
+      <c r="M18" s="50"/>
+      <c r="N18" s="50"/>
+      <c r="O18" s="156"/>
+      <c r="P18" s="155"/>
+    </row>
+    <row r="19" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A19" s="78"/>
+      <c r="B19" s="80"/>
       <c r="C19" s="42"/>
       <c r="D19" s="42"/>
       <c r="E19" s="42"/>
       <c r="F19" s="42"/>
-      <c r="G19" s="57"/>
-      <c r="H19" s="77"/>
-      <c r="I19" s="77"/>
+      <c r="G19" s="55"/>
+      <c r="H19" s="73"/>
+      <c r="I19" s="73"/>
       <c r="J19" s="42"/>
-      <c r="K19" s="52"/>
-      <c r="L19" s="52"/>
-      <c r="M19" s="52"/>
-      <c r="N19" s="52"/>
-      <c r="O19" s="78"/>
-      <c r="P19" s="63"/>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A20" s="83"/>
-      <c r="B20" s="85"/>
+      <c r="K19" s="50"/>
+      <c r="L19" s="50"/>
+      <c r="M19" s="50"/>
+      <c r="N19" s="50"/>
+      <c r="O19" s="154"/>
+      <c r="P19" s="155"/>
+    </row>
+    <row r="20" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A20" s="78"/>
+      <c r="B20" s="80"/>
       <c r="C20" s="42"/>
       <c r="D20" s="42"/>
       <c r="E20" s="42"/>
       <c r="F20" s="42"/>
-      <c r="G20" s="57"/>
+      <c r="G20" s="55"/>
       <c r="H20" s="42"/>
       <c r="I20" s="42"/>
       <c r="J20" s="42"/>
-      <c r="K20" s="52"/>
-      <c r="L20" s="52"/>
-      <c r="M20" s="52"/>
-      <c r="N20" s="52"/>
-      <c r="O20" s="46"/>
-      <c r="P20" s="63"/>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A21" s="83"/>
-      <c r="B21" s="85"/>
+      <c r="K20" s="50"/>
+      <c r="L20" s="50"/>
+      <c r="M20" s="50"/>
+      <c r="N20" s="50"/>
+      <c r="O20" s="156"/>
+      <c r="P20" s="155"/>
+    </row>
+    <row r="21" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A21" s="78"/>
+      <c r="B21" s="80"/>
       <c r="C21" s="42"/>
       <c r="D21" s="42"/>
       <c r="E21" s="42"/>
       <c r="F21" s="42"/>
-      <c r="G21" s="57"/>
+      <c r="G21" s="55"/>
       <c r="H21" s="42"/>
       <c r="I21" s="42"/>
       <c r="J21" s="42"/>
-      <c r="K21" s="52"/>
-      <c r="L21" s="52"/>
-      <c r="M21" s="52"/>
-      <c r="N21" s="52"/>
-      <c r="O21" s="46"/>
-      <c r="P21" s="63"/>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A22" s="83"/>
-      <c r="B22" s="85"/>
+      <c r="K21" s="50"/>
+      <c r="L21" s="50"/>
+      <c r="M21" s="50"/>
+      <c r="N21" s="50"/>
+      <c r="O21" s="156"/>
+      <c r="P21" s="155"/>
+    </row>
+    <row r="22" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A22" s="78"/>
+      <c r="B22" s="80"/>
       <c r="C22" s="42"/>
       <c r="D22" s="42"/>
       <c r="E22" s="42"/>
       <c r="F22" s="42"/>
-      <c r="G22" s="57"/>
-      <c r="H22" s="77"/>
-      <c r="I22" s="77"/>
+      <c r="G22" s="55"/>
+      <c r="H22" s="73"/>
+      <c r="I22" s="73"/>
       <c r="J22" s="42"/>
-      <c r="K22" s="52"/>
-      <c r="L22" s="52"/>
-      <c r="M22" s="52"/>
-      <c r="N22" s="52"/>
-      <c r="O22" s="46"/>
-      <c r="P22" s="63"/>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A23" s="83"/>
-      <c r="B23" s="85"/>
+      <c r="K22" s="50"/>
+      <c r="L22" s="50"/>
+      <c r="M22" s="50"/>
+      <c r="N22" s="50"/>
+      <c r="O22" s="156"/>
+      <c r="P22" s="155"/>
+    </row>
+    <row r="23" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A23" s="78"/>
+      <c r="B23" s="80"/>
       <c r="C23" s="42"/>
       <c r="D23" s="42"/>
       <c r="E23" s="42"/>
       <c r="F23" s="42"/>
-      <c r="G23" s="57"/>
-      <c r="H23" s="77"/>
-      <c r="I23" s="77"/>
+      <c r="G23" s="55"/>
+      <c r="H23" s="73"/>
+      <c r="I23" s="73"/>
       <c r="J23" s="42"/>
-      <c r="K23" s="52"/>
-      <c r="L23" s="52"/>
-      <c r="M23" s="52"/>
-      <c r="N23" s="52"/>
-      <c r="O23" s="46"/>
-      <c r="P23" s="63"/>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A24" s="62"/>
-      <c r="B24" s="51"/>
+      <c r="K23" s="50"/>
+      <c r="L23" s="50"/>
+      <c r="M23" s="50"/>
+      <c r="N23" s="50"/>
+      <c r="O23" s="156"/>
+      <c r="P23" s="155"/>
+    </row>
+    <row r="24" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A24" s="60"/>
+      <c r="B24" s="49"/>
       <c r="C24" s="42"/>
       <c r="D24" s="42"/>
       <c r="E24" s="42"/>
       <c r="F24" s="42"/>
-      <c r="G24" s="57"/>
-      <c r="H24" s="77"/>
-      <c r="I24" s="77"/>
+      <c r="G24" s="55"/>
+      <c r="H24" s="73"/>
+      <c r="I24" s="73"/>
       <c r="J24" s="42"/>
-      <c r="K24" s="52"/>
-      <c r="L24" s="52"/>
-      <c r="M24" s="52"/>
-      <c r="N24" s="52"/>
-      <c r="O24" s="46"/>
-      <c r="P24" s="63"/>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A25" s="62"/>
-      <c r="B25" s="51"/>
+      <c r="K24" s="50"/>
+      <c r="L24" s="50"/>
+      <c r="M24" s="50"/>
+      <c r="N24" s="50"/>
+      <c r="O24" s="156"/>
+      <c r="P24" s="155"/>
+    </row>
+    <row r="25" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A25" s="60"/>
+      <c r="B25" s="49"/>
       <c r="C25" s="42"/>
       <c r="D25" s="42"/>
       <c r="E25" s="42"/>
       <c r="F25" s="42"/>
-      <c r="G25" s="57"/>
-      <c r="H25" s="77"/>
-      <c r="I25" s="77"/>
+      <c r="G25" s="55"/>
+      <c r="H25" s="73"/>
+      <c r="I25" s="73"/>
       <c r="J25" s="42"/>
-      <c r="K25" s="52"/>
-      <c r="L25" s="52"/>
-      <c r="M25" s="52"/>
-      <c r="N25" s="52"/>
-      <c r="O25" s="46"/>
-      <c r="P25" s="63"/>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A26" s="62"/>
-      <c r="B26" s="51"/>
+      <c r="K25" s="50"/>
+      <c r="L25" s="50"/>
+      <c r="M25" s="50"/>
+      <c r="N25" s="50"/>
+      <c r="O25" s="156"/>
+      <c r="P25" s="155"/>
+    </row>
+    <row r="26" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A26" s="60"/>
+      <c r="B26" s="49"/>
       <c r="C26" s="42"/>
       <c r="D26" s="42"/>
       <c r="E26" s="42"/>
       <c r="F26" s="42"/>
-      <c r="G26" s="57"/>
-      <c r="H26" s="77"/>
-      <c r="I26" s="77"/>
+      <c r="G26" s="55"/>
+      <c r="H26" s="73"/>
+      <c r="I26" s="73"/>
       <c r="J26" s="42"/>
-      <c r="K26" s="52"/>
-      <c r="L26" s="52"/>
-      <c r="M26" s="52"/>
-      <c r="N26" s="52"/>
-      <c r="O26" s="46"/>
-      <c r="P26" s="63"/>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A27" s="62"/>
-      <c r="B27" s="51"/>
+      <c r="K26" s="50"/>
+      <c r="L26" s="50"/>
+      <c r="M26" s="50"/>
+      <c r="N26" s="50"/>
+      <c r="O26" s="156"/>
+      <c r="P26" s="155"/>
+    </row>
+    <row r="27" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A27" s="60"/>
+      <c r="B27" s="49"/>
       <c r="C27" s="42"/>
       <c r="D27" s="42"/>
       <c r="E27" s="42"/>
       <c r="F27" s="42"/>
-      <c r="G27" s="57"/>
+      <c r="G27" s="55"/>
       <c r="H27" s="42"/>
       <c r="I27" s="42"/>
       <c r="J27" s="42"/>
-      <c r="K27" s="52"/>
-      <c r="L27" s="52"/>
-      <c r="M27" s="52"/>
-      <c r="N27" s="52"/>
-      <c r="O27" s="46"/>
-      <c r="P27" s="63"/>
-      <c r="Q27" s="49"/>
-      <c r="R27" s="49"/>
-    </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A28" s="64"/>
-      <c r="B28" s="51"/>
-      <c r="C28" s="51"/>
+      <c r="K27" s="50"/>
+      <c r="L27" s="50"/>
+      <c r="M27" s="50"/>
+      <c r="N27" s="50"/>
+      <c r="O27" s="156"/>
+      <c r="P27" s="155"/>
+      <c r="Q27" s="48"/>
+      <c r="R27" s="48"/>
+    </row>
+    <row r="28" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A28" s="61"/>
+      <c r="B28" s="49"/>
+      <c r="C28" s="49"/>
       <c r="D28" s="42">
         <f>SUM(D8:D27)</f>
         <v>0</v>
@@ -3343,149 +3352,161 @@
       <c r="F28" s="42"/>
       <c r="G28" s="42"/>
       <c r="H28" s="42"/>
-      <c r="I28" s="57"/>
+      <c r="I28" s="55"/>
       <c r="J28" s="42"/>
-      <c r="K28" s="69">
+      <c r="K28" s="65">
         <f>SUM(K8:K27)</f>
         <v>0</v>
       </c>
-      <c r="L28" s="69">
+      <c r="L28" s="65">
         <f>SUM(L8:L27)</f>
         <v>0</v>
       </c>
-      <c r="M28" s="69">
+      <c r="M28" s="65">
         <f>SUM(M8:M27)</f>
         <v>0</v>
       </c>
-      <c r="N28" s="69">
+      <c r="N28" s="65">
         <f>SUM(N8:N27)</f>
         <v>0</v>
       </c>
-      <c r="O28" s="50"/>
-      <c r="P28" s="65"/>
-      <c r="Q28" s="48"/>
-      <c r="R28" s="49"/>
-    </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A29" s="66" t="s">
+      <c r="O28" s="157"/>
+      <c r="P28" s="158"/>
+      <c r="Q28" s="47"/>
+      <c r="R28" s="48"/>
+    </row>
+    <row r="29" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A29" s="62" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="126">
+      <c r="B29" s="139">
         <f>B30+F30</f>
         <v>0</v>
       </c>
-      <c r="C29" s="127"/>
-      <c r="D29" s="128"/>
-      <c r="E29" s="47" t="s">
+      <c r="C29" s="140"/>
+      <c r="D29" s="141"/>
+      <c r="E29" s="46" t="s">
         <v>30</v>
       </c>
-      <c r="F29" s="47"/>
-      <c r="G29" s="47"/>
-      <c r="H29" s="112" t="s">
+      <c r="F29" s="46"/>
+      <c r="G29" s="46"/>
+      <c r="H29" s="125" t="s">
         <v>33</v>
       </c>
-      <c r="I29" s="113"/>
-      <c r="J29" s="114"/>
-      <c r="K29" s="132">
+      <c r="I29" s="126"/>
+      <c r="J29" s="127"/>
+      <c r="K29" s="145">
         <f>B31</f>
         <v>0</v>
       </c>
-      <c r="L29" s="133"/>
-      <c r="M29" s="133"/>
-      <c r="N29" s="133"/>
-      <c r="O29" s="133"/>
-      <c r="P29" s="134"/>
-      <c r="Q29" s="48"/>
-      <c r="R29" s="49"/>
-    </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A30" s="66" t="s">
+      <c r="L29" s="146"/>
+      <c r="M29" s="146"/>
+      <c r="N29" s="146"/>
+      <c r="O29" s="146"/>
+      <c r="P29" s="147"/>
+      <c r="Q29" s="47"/>
+      <c r="R29" s="48"/>
+    </row>
+    <row r="30" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A30" s="62" t="s">
         <v>40</v>
       </c>
-      <c r="B30" s="129">
+      <c r="B30" s="142">
         <f>L28</f>
         <v>0</v>
       </c>
-      <c r="C30" s="130"/>
-      <c r="D30" s="131"/>
-      <c r="E30" s="47" t="s">
+      <c r="C30" s="143"/>
+      <c r="D30" s="144"/>
+      <c r="E30" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="F30" s="129">
+      <c r="F30" s="142">
         <f>M28+N28</f>
         <v>0</v>
       </c>
-      <c r="G30" s="131"/>
-      <c r="H30" s="115"/>
-      <c r="I30" s="116"/>
-      <c r="J30" s="117"/>
-      <c r="K30" s="135"/>
-      <c r="L30" s="136"/>
-      <c r="M30" s="136"/>
-      <c r="N30" s="136"/>
-      <c r="O30" s="136"/>
-      <c r="P30" s="137"/>
-      <c r="Q30" s="48"/>
-      <c r="R30" s="49"/>
-    </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A31" s="66" t="s">
+      <c r="G30" s="144"/>
+      <c r="H30" s="128"/>
+      <c r="I30" s="129"/>
+      <c r="J30" s="130"/>
+      <c r="K30" s="148"/>
+      <c r="L30" s="149"/>
+      <c r="M30" s="149"/>
+      <c r="N30" s="149"/>
+      <c r="O30" s="149"/>
+      <c r="P30" s="150"/>
+      <c r="Q30" s="47"/>
+      <c r="R30" s="48"/>
+    </row>
+    <row r="31" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A31" s="62" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="121">
+      <c r="B31" s="134">
         <f>K28</f>
         <v>0</v>
       </c>
-      <c r="C31" s="122"/>
-      <c r="D31" s="123"/>
-      <c r="E31" s="58" t="s">
+      <c r="C31" s="135"/>
+      <c r="D31" s="136"/>
+      <c r="E31" s="56" t="s">
         <v>36</v>
       </c>
-      <c r="F31" s="110">
+      <c r="F31" s="123">
         <f>D28</f>
         <v>0</v>
       </c>
-      <c r="G31" s="111"/>
-      <c r="H31" s="115"/>
-      <c r="I31" s="116"/>
-      <c r="J31" s="117"/>
-      <c r="K31" s="135"/>
-      <c r="L31" s="136"/>
-      <c r="M31" s="136"/>
-      <c r="N31" s="136"/>
-      <c r="O31" s="136"/>
-      <c r="P31" s="137"/>
-      <c r="Q31" s="48"/>
-      <c r="R31" s="49"/>
-    </row>
-    <row r="32" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="67" t="s">
+      <c r="G31" s="124"/>
+      <c r="H31" s="128"/>
+      <c r="I31" s="129"/>
+      <c r="J31" s="130"/>
+      <c r="K31" s="148"/>
+      <c r="L31" s="149"/>
+      <c r="M31" s="149"/>
+      <c r="N31" s="149"/>
+      <c r="O31" s="149"/>
+      <c r="P31" s="150"/>
+      <c r="Q31" s="47"/>
+      <c r="R31" s="48"/>
+    </row>
+    <row r="32" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="63" t="s">
         <v>38</v>
       </c>
-      <c r="B32" s="68"/>
-      <c r="C32" s="124">
+      <c r="B32" s="64"/>
+      <c r="C32" s="137">
         <v>0</v>
       </c>
-      <c r="D32" s="125"/>
-      <c r="E32" s="68" t="s">
+      <c r="D32" s="138"/>
+      <c r="E32" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="F32" s="68"/>
-      <c r="G32" s="68"/>
-      <c r="H32" s="118"/>
-      <c r="I32" s="119"/>
-      <c r="J32" s="120"/>
-      <c r="K32" s="138"/>
-      <c r="L32" s="139"/>
-      <c r="M32" s="139"/>
-      <c r="N32" s="139"/>
-      <c r="O32" s="139"/>
-      <c r="P32" s="140"/>
-      <c r="Q32" s="49"/>
-      <c r="R32" s="49"/>
+      <c r="F32" s="64"/>
+      <c r="G32" s="64"/>
+      <c r="H32" s="131"/>
+      <c r="I32" s="132"/>
+      <c r="J32" s="133"/>
+      <c r="K32" s="151"/>
+      <c r="L32" s="152"/>
+      <c r="M32" s="152"/>
+      <c r="N32" s="152"/>
+      <c r="O32" s="152"/>
+      <c r="P32" s="153"/>
+      <c r="Q32" s="48"/>
+      <c r="R32" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="H29:J32"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="K29:P32"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="E3:I3"/>
     <mergeCell ref="Q5:R5"/>
     <mergeCell ref="J3:K3"/>
     <mergeCell ref="A4:C4"/>
@@ -3502,18 +3523,6 @@
     <mergeCell ref="K5:K7"/>
     <mergeCell ref="J5:J7"/>
     <mergeCell ref="E5:E7"/>
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="H29:J32"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="K29:P32"/>
-    <mergeCell ref="D5:D7"/>
-    <mergeCell ref="E3:I3"/>
   </mergeCells>
   <phoneticPr fontId="27" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update: Refactor database management UI and enhance data cleaning functionality
- Improved the database management page layout for better user experience, including adjustments to tab organization and button placements.
- Integrated a new feature to remove database files to the recycle bin, enhancing data management capabilities.
- Updated the `clean_database_data` function to provide detailed logging of the cleaning process and return structured results, improving feedback to users.
- Refactored various UI components for consistency and clarity in user interactions.
</commit_message>
<xml_diff>
--- a/resources/Out_format.xlsx
+++ b/resources/Out_format.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\my_github\FlightCheckPy\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{950BD087-C01E-4909-BA88-E013711A771D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F236E3F5-F285-49E2-AAB9-EAA8717609E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{D6DB75D4-A8CC-4A73-9AF5-6E324AED1BA5}"/>
+    <workbookView xWindow="5625" yWindow="4815" windowWidth="18750" windowHeight="15345" activeTab="1" xr2:uid="{D6DB75D4-A8CC-4A73-9AF5-6E324AED1BA5}"/>
   </bookViews>
   <sheets>
     <sheet name="RECEIPT" sheetId="17" r:id="rId1"/>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="82">
   <si>
     <t>AIR CHINA MISCELLANEOUS CHARGES ORDER SALES REPORT</t>
   </si>
@@ -441,6 +441,10 @@
   </si>
   <si>
     <t>CA</t>
+  </si>
+  <si>
+    <t>No Cash</t>
+    <phoneticPr fontId="40" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1272,6 +1276,45 @@
     <xf numFmtId="1" fontId="9" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="181" fontId="9" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="9" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="9" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="distributed"/>
     </xf>
@@ -1281,15 +1324,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1301,27 +1335,6 @@
     </xf>
     <xf numFmtId="178" fontId="22" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1340,13 +1353,118 @@
     <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="10" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="28" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="26" fontId="3" fillId="0" borderId="10" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1357,12 +1475,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1391,119 +1503,11 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="10" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="9" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="9" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="14">
@@ -2009,11 +2013,11 @@
     <row r="2" spans="1:12" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="C2" s="3"/>
-      <c r="D2" s="81" t="s">
+      <c r="D2" s="94" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81"/>
+      <c r="E2" s="94"/>
+      <c r="F2" s="94"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="25"/>
@@ -2022,16 +2026,16 @@
       <c r="A3" s="32"/>
       <c r="B3" s="32"/>
       <c r="C3" s="32"/>
-      <c r="D3" s="82" t="s">
+      <c r="D3" s="95" t="s">
         <v>45</v>
       </c>
-      <c r="E3" s="82"/>
-      <c r="F3" s="82"/>
-      <c r="G3" s="83" t="s">
+      <c r="E3" s="95"/>
+      <c r="F3" s="95"/>
+      <c r="G3" s="96" t="s">
         <v>46</v>
       </c>
-      <c r="H3" s="83"/>
-      <c r="I3" s="83"/>
+      <c r="H3" s="96"/>
+      <c r="I3" s="96"/>
       <c r="J3" s="35"/>
       <c r="K3" s="35"/>
       <c r="L3" s="34"/>
@@ -2050,198 +2054,200 @@
       <c r="K4" s="24"/>
     </row>
     <row r="5" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="84" t="s">
+      <c r="A5" s="89" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="84"/>
-      <c r="C5" s="85">
+      <c r="B5" s="89"/>
+      <c r="C5" s="86">
         <f>SUM!C13</f>
         <v>0</v>
       </c>
-      <c r="D5" s="85"/>
-      <c r="E5" s="85"/>
-      <c r="F5" s="87" t="s">
+      <c r="D5" s="86"/>
+      <c r="E5" s="86"/>
+      <c r="F5" s="97" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="89">
+      <c r="G5" s="99">
         <f>SUM!G11</f>
         <v>0</v>
       </c>
-      <c r="H5" s="89"/>
-      <c r="I5" s="89"/>
+      <c r="H5" s="99"/>
+      <c r="I5" s="99"/>
       <c r="J5" s="33"/>
       <c r="K5" s="33"/>
     </row>
     <row r="6" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="91" t="s">
+      <c r="A6" s="90" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="91"/>
-      <c r="C6" s="86"/>
-      <c r="D6" s="86"/>
-      <c r="E6" s="86"/>
-      <c r="F6" s="88"/>
-      <c r="G6" s="90"/>
-      <c r="H6" s="90"/>
-      <c r="I6" s="90"/>
+      <c r="B6" s="90"/>
+      <c r="C6" s="87"/>
+      <c r="D6" s="87"/>
+      <c r="E6" s="87"/>
+      <c r="F6" s="98"/>
+      <c r="G6" s="100"/>
+      <c r="H6" s="100"/>
+      <c r="I6" s="100"/>
       <c r="J6" s="33"/>
       <c r="K6" s="33"/>
     </row>
     <row r="8" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="92" t="s">
+      <c r="A8" s="93" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="92"/>
-      <c r="C8" s="93"/>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
+      <c r="B8" s="93"/>
+      <c r="C8" s="157" t="s">
+        <v>81</v>
+      </c>
+      <c r="D8" s="157"/>
+      <c r="E8" s="157"/>
+      <c r="F8" s="157"/>
+      <c r="G8" s="157"/>
+      <c r="H8" s="157"/>
+      <c r="I8" s="157"/>
     </row>
     <row r="9" spans="1:12" ht="49.7" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="92"/>
-      <c r="B9" s="92"/>
-      <c r="C9" s="94"/>
-      <c r="D9" s="94"/>
-      <c r="E9" s="94"/>
-      <c r="F9" s="94"/>
-      <c r="G9" s="94"/>
-      <c r="H9" s="94"/>
-      <c r="I9" s="94"/>
+      <c r="A9" s="93"/>
+      <c r="B9" s="93"/>
+      <c r="C9" s="158"/>
+      <c r="D9" s="158"/>
+      <c r="E9" s="158"/>
+      <c r="F9" s="158"/>
+      <c r="G9" s="158"/>
+      <c r="H9" s="158"/>
+      <c r="I9" s="158"/>
     </row>
     <row r="11" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A11" s="84" t="s">
+      <c r="A11" s="89" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="84"/>
-      <c r="C11" s="85" t="s">
+      <c r="B11" s="89"/>
+      <c r="C11" s="86" t="s">
         <v>50</v>
       </c>
-      <c r="D11" s="85"/>
-      <c r="E11" s="85"/>
+      <c r="D11" s="86"/>
+      <c r="E11" s="86"/>
       <c r="F11" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="G11" s="95">
+      <c r="G11" s="88">
         <f>SUM!C14</f>
         <v>0</v>
       </c>
-      <c r="H11" s="85"/>
-      <c r="I11" s="85"/>
+      <c r="H11" s="86"/>
+      <c r="I11" s="86"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" s="91" t="s">
+      <c r="A12" s="90" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="91"/>
-      <c r="C12" s="86"/>
-      <c r="D12" s="86"/>
-      <c r="E12" s="86"/>
+      <c r="B12" s="90"/>
+      <c r="C12" s="87"/>
+      <c r="D12" s="87"/>
+      <c r="E12" s="87"/>
       <c r="F12" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="G12" s="86"/>
-      <c r="H12" s="86"/>
-      <c r="I12" s="86"/>
+      <c r="G12" s="87"/>
+      <c r="H12" s="87"/>
+      <c r="I12" s="87"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" s="84" t="s">
+      <c r="A14" s="89" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="84"/>
-      <c r="C14" s="85" t="s">
+      <c r="B14" s="89"/>
+      <c r="C14" s="86" t="s">
         <v>78</v>
       </c>
-      <c r="D14" s="85"/>
-      <c r="E14" s="85"/>
-      <c r="F14" s="85"/>
-      <c r="G14" s="85"/>
-      <c r="H14" s="85"/>
-      <c r="I14" s="85"/>
+      <c r="D14" s="86"/>
+      <c r="E14" s="86"/>
+      <c r="F14" s="86"/>
+      <c r="G14" s="86"/>
+      <c r="H14" s="86"/>
+      <c r="I14" s="86"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A15" s="91" t="s">
+      <c r="A15" s="90" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="91"/>
-      <c r="C15" s="86"/>
-      <c r="D15" s="86"/>
-      <c r="E15" s="86"/>
-      <c r="F15" s="86"/>
-      <c r="G15" s="86"/>
-      <c r="H15" s="86"/>
-      <c r="I15" s="86"/>
+      <c r="B15" s="90"/>
+      <c r="C15" s="87"/>
+      <c r="D15" s="87"/>
+      <c r="E15" s="87"/>
+      <c r="F15" s="87"/>
+      <c r="G15" s="87"/>
+      <c r="H15" s="87"/>
+      <c r="I15" s="87"/>
     </row>
     <row r="17" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="B17" s="85" t="s">
+      <c r="B17" s="86" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="85"/>
-      <c r="D17" s="85"/>
-      <c r="E17" s="85"/>
+      <c r="C17" s="86"/>
+      <c r="D17" s="86"/>
+      <c r="E17" s="86"/>
       <c r="F17" s="31" t="s">
         <v>58</v>
       </c>
       <c r="G17" s="31"/>
-      <c r="H17" s="85" t="s">
+      <c r="H17" s="86" t="s">
         <v>59</v>
       </c>
-      <c r="I17" s="85"/>
+      <c r="I17" s="86"/>
     </row>
     <row r="18" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
         <v>60</v>
       </c>
-      <c r="B18" s="86"/>
-      <c r="C18" s="86"/>
-      <c r="D18" s="86"/>
-      <c r="E18" s="86"/>
-      <c r="F18" s="96" t="s">
+      <c r="B18" s="87"/>
+      <c r="C18" s="87"/>
+      <c r="D18" s="87"/>
+      <c r="E18" s="87"/>
+      <c r="F18" s="91" t="s">
         <v>61</v>
       </c>
-      <c r="G18" s="97"/>
-      <c r="H18" s="86"/>
-      <c r="I18" s="86"/>
+      <c r="G18" s="92"/>
+      <c r="H18" s="87"/>
+      <c r="I18" s="87"/>
     </row>
     <row r="20" spans="1:9" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="B20" s="85" t="s">
+      <c r="B20" s="86" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="85"/>
-      <c r="D20" s="85"/>
-      <c r="E20" s="85"/>
+      <c r="C20" s="86"/>
+      <c r="D20" s="86"/>
+      <c r="E20" s="86"/>
       <c r="F20" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="G20" s="95">
+      <c r="G20" s="88">
         <f>SUM!C14</f>
         <v>0</v>
       </c>
-      <c r="H20" s="85"/>
-      <c r="I20" s="85"/>
+      <c r="H20" s="86"/>
+      <c r="I20" s="86"/>
     </row>
     <row r="21" spans="1:9" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="B21" s="86"/>
-      <c r="C21" s="86"/>
-      <c r="D21" s="86"/>
-      <c r="E21" s="86"/>
+      <c r="B21" s="87"/>
+      <c r="C21" s="87"/>
+      <c r="D21" s="87"/>
+      <c r="E21" s="87"/>
       <c r="F21" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="G21" s="86"/>
-      <c r="H21" s="86"/>
-      <c r="I21" s="86"/>
+      <c r="G21" s="87"/>
+      <c r="H21" s="87"/>
+      <c r="I21" s="87"/>
     </row>
     <row r="22" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A22" s="27"/>
@@ -2269,6 +2275,20 @@
     <row r="47" ht="13.15" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="G5:I6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A8:B9"/>
+    <mergeCell ref="C8:I9"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:E12"/>
+    <mergeCell ref="G11:I12"/>
+    <mergeCell ref="A12:B12"/>
     <mergeCell ref="B20:E21"/>
     <mergeCell ref="G20:I21"/>
     <mergeCell ref="A14:B14"/>
@@ -2277,20 +2297,6 @@
     <mergeCell ref="B17:E18"/>
     <mergeCell ref="H17:I18"/>
     <mergeCell ref="F18:G18"/>
-    <mergeCell ref="A8:B9"/>
-    <mergeCell ref="C8:I9"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:E12"/>
-    <mergeCell ref="G11:I12"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="G5:I6"/>
-    <mergeCell ref="A6:B6"/>
   </mergeCells>
   <phoneticPr fontId="40" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2352,19 +2358,19 @@
       <c r="K2" s="25"/>
     </row>
     <row r="3" spans="1:14" ht="19.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="101" t="s">
+      <c r="A3" s="104" t="s">
         <v>74</v>
       </c>
-      <c r="B3" s="101"/>
-      <c r="C3" s="101"/>
-      <c r="D3" s="101"/>
-      <c r="E3" s="101"/>
-      <c r="F3" s="101"/>
-      <c r="G3" s="101"/>
-      <c r="H3" s="101"/>
-      <c r="I3" s="101"/>
-      <c r="J3" s="101"/>
-      <c r="K3" s="101"/>
+      <c r="B3" s="104"/>
+      <c r="C3" s="104"/>
+      <c r="D3" s="104"/>
+      <c r="E3" s="104"/>
+      <c r="F3" s="104"/>
+      <c r="G3" s="104"/>
+      <c r="H3" s="104"/>
+      <c r="I3" s="104"/>
+      <c r="J3" s="104"/>
+      <c r="K3" s="104"/>
       <c r="L3" s="23"/>
       <c r="M3" s="23"/>
       <c r="N3" s="23"/>
@@ -2421,32 +2427,32 @@
     </row>
     <row r="7" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="21"/>
-      <c r="B7" s="104" t="s">
+      <c r="B7" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="98" t="s">
+      <c r="C7" s="101" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="98" t="s">
+      <c r="D7" s="101" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="98" t="s">
+      <c r="E7" s="101" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="98" t="s">
+      <c r="F7" s="101" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="98" t="s">
+      <c r="G7" s="101" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="102" t="s">
+      <c r="H7" s="105" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="103"/>
-      <c r="J7" s="98" t="s">
+      <c r="I7" s="106"/>
+      <c r="J7" s="101" t="s">
         <v>10</v>
       </c>
-      <c r="K7" s="98" t="s">
+      <c r="K7" s="101" t="s">
         <v>9</v>
       </c>
       <c r="L7" s="2"/>
@@ -2454,20 +2460,20 @@
     </row>
     <row r="8" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="21"/>
-      <c r="B8" s="104"/>
-      <c r="C8" s="98"/>
-      <c r="D8" s="98"/>
-      <c r="E8" s="98"/>
-      <c r="F8" s="98"/>
-      <c r="G8" s="98"/>
+      <c r="B8" s="107"/>
+      <c r="C8" s="101"/>
+      <c r="D8" s="101"/>
+      <c r="E8" s="101"/>
+      <c r="F8" s="101"/>
+      <c r="G8" s="101"/>
       <c r="H8" s="20" t="s">
         <v>8</v>
       </c>
       <c r="I8" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="J8" s="98"/>
-      <c r="K8" s="98"/>
+      <c r="J8" s="101"/>
+      <c r="K8" s="101"/>
       <c r="L8" s="2"/>
       <c r="M8" s="8"/>
     </row>
@@ -2703,8 +2709,8 @@
       <c r="K20" s="3"/>
     </row>
     <row r="21" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="C21" s="99"/>
-      <c r="D21" s="100"/>
+      <c r="C21" s="102"/>
+      <c r="D21" s="103"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C22" s="2"/>
@@ -2780,47 +2786,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="121" t="s">
+      <c r="A1" s="108" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="121"/>
-      <c r="C1" s="121"/>
-      <c r="D1" s="121"/>
-      <c r="E1" s="121"/>
-      <c r="F1" s="121"/>
-      <c r="G1" s="121"/>
-      <c r="H1" s="121"/>
-      <c r="I1" s="121"/>
-      <c r="J1" s="121"/>
-      <c r="K1" s="121"/>
-      <c r="L1" s="121"/>
-      <c r="M1" s="121"/>
-      <c r="N1" s="121"/>
-      <c r="O1" s="121"/>
-      <c r="P1" s="121"/>
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="108"/>
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="108"/>
+      <c r="L1" s="108"/>
+      <c r="M1" s="108"/>
+      <c r="N1" s="108"/>
+      <c r="O1" s="108"/>
+      <c r="P1" s="108"/>
       <c r="Q1" s="68"/>
       <c r="R1" s="68"/>
       <c r="S1" s="68"/>
     </row>
     <row r="2" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="122" t="s">
+      <c r="A2" s="109" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="122"/>
-      <c r="C2" s="122"/>
-      <c r="D2" s="122"/>
-      <c r="E2" s="122"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="122"/>
-      <c r="H2" s="122"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="122"/>
-      <c r="K2" s="122"/>
-      <c r="L2" s="122"/>
-      <c r="M2" s="122"/>
-      <c r="N2" s="122"/>
-      <c r="O2" s="122"/>
-      <c r="P2" s="122"/>
+      <c r="B2" s="109"/>
+      <c r="C2" s="109"/>
+      <c r="D2" s="109"/>
+      <c r="E2" s="109"/>
+      <c r="F2" s="109"/>
+      <c r="G2" s="109"/>
+      <c r="H2" s="109"/>
+      <c r="I2" s="109"/>
+      <c r="J2" s="109"/>
+      <c r="K2" s="109"/>
+      <c r="L2" s="109"/>
+      <c r="M2" s="109"/>
+      <c r="N2" s="109"/>
+      <c r="O2" s="109"/>
+      <c r="P2" s="109"/>
       <c r="Q2" s="69"/>
       <c r="R2" s="69"/>
       <c r="S2" s="69"/>
@@ -2831,18 +2837,18 @@
       </c>
       <c r="B3" s="44"/>
       <c r="C3" s="44"/>
-      <c r="E3" s="106" t="str">
+      <c r="E3" s="143" t="str">
         <f>"报告期间：" &amp; N3 &amp; "至" &amp; N3</f>
         <v>报告期间：1900年1月0日至1900年1月0日</v>
       </c>
-      <c r="F3" s="106"/>
-      <c r="G3" s="106"/>
-      <c r="H3" s="106"/>
-      <c r="I3" s="106"/>
-      <c r="J3" s="106" t="s">
+      <c r="F3" s="143"/>
+      <c r="G3" s="143"/>
+      <c r="H3" s="143"/>
+      <c r="I3" s="143"/>
+      <c r="J3" s="143" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="106"/>
+      <c r="K3" s="143"/>
       <c r="L3" s="43"/>
       <c r="M3" s="66"/>
       <c r="N3" s="66" t="str">
@@ -2856,17 +2862,17 @@
       <c r="S3" s="45"/>
     </row>
     <row r="4" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="107" t="s">
+      <c r="A4" s="145" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="107"/>
-      <c r="C4" s="107"/>
+      <c r="B4" s="145"/>
+      <c r="C4" s="145"/>
       <c r="D4" s="70"/>
       <c r="E4" s="70"/>
       <c r="F4" s="71"/>
       <c r="G4" s="72"/>
-      <c r="H4" s="108"/>
-      <c r="I4" s="108"/>
+      <c r="H4" s="146"/>
+      <c r="I4" s="146"/>
       <c r="J4" s="67" t="s">
         <v>76</v>
       </c>
@@ -2881,68 +2887,68 @@
       <c r="P4" s="67"/>
     </row>
     <row r="5" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="119" t="s">
+      <c r="A5" s="155" t="s">
         <v>70</v>
       </c>
-      <c r="B5" s="117" t="s">
+      <c r="B5" s="153" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="115" t="s">
+      <c r="C5" s="151" t="s">
         <v>72</v>
       </c>
-      <c r="D5" s="111" t="s">
+      <c r="D5" s="141" t="s">
         <v>73</v>
       </c>
-      <c r="E5" s="109" t="s">
+      <c r="E5" s="147" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="111" t="s">
+      <c r="F5" s="141" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="109" t="s">
+      <c r="G5" s="147" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="109" t="s">
+      <c r="H5" s="147" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="109" t="s">
+      <c r="I5" s="147" t="s">
         <v>28</v>
       </c>
-      <c r="J5" s="109" t="s">
+      <c r="J5" s="147" t="s">
         <v>29</v>
       </c>
-      <c r="K5" s="111" t="s">
+      <c r="K5" s="141" t="s">
         <v>24</v>
       </c>
-      <c r="L5" s="113" t="s">
+      <c r="L5" s="149" t="s">
         <v>41</v>
       </c>
-      <c r="M5" s="113" t="s">
+      <c r="M5" s="149" t="s">
         <v>42</v>
       </c>
-      <c r="N5" s="113"/>
+      <c r="N5" s="149"/>
       <c r="O5" s="57" t="s">
         <v>66</v>
       </c>
       <c r="P5" s="58" t="s">
         <v>67</v>
       </c>
-      <c r="Q5" s="105"/>
-      <c r="R5" s="105"/>
+      <c r="Q5" s="144"/>
+      <c r="R5" s="144"/>
     </row>
     <row r="6" spans="1:19" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="120"/>
-      <c r="B6" s="118"/>
-      <c r="C6" s="116"/>
-      <c r="D6" s="112"/>
-      <c r="E6" s="110"/>
-      <c r="F6" s="112"/>
-      <c r="G6" s="110"/>
-      <c r="H6" s="110"/>
-      <c r="I6" s="110"/>
-      <c r="J6" s="110"/>
-      <c r="K6" s="112"/>
-      <c r="L6" s="114"/>
+      <c r="A6" s="156"/>
+      <c r="B6" s="154"/>
+      <c r="C6" s="152"/>
+      <c r="D6" s="142"/>
+      <c r="E6" s="148"/>
+      <c r="F6" s="142"/>
+      <c r="G6" s="148"/>
+      <c r="H6" s="148"/>
+      <c r="I6" s="148"/>
+      <c r="J6" s="148"/>
+      <c r="K6" s="142"/>
+      <c r="L6" s="150"/>
       <c r="M6" s="53" t="s">
         <v>43</v>
       </c>
@@ -2957,17 +2963,17 @@
       </c>
     </row>
     <row r="7" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A7" s="120"/>
-      <c r="B7" s="118"/>
-      <c r="C7" s="116"/>
-      <c r="D7" s="112"/>
-      <c r="E7" s="110"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="110"/>
-      <c r="H7" s="110"/>
-      <c r="I7" s="110"/>
-      <c r="J7" s="110"/>
-      <c r="K7" s="112"/>
+      <c r="A7" s="156"/>
+      <c r="B7" s="154"/>
+      <c r="C7" s="152"/>
+      <c r="D7" s="142"/>
+      <c r="E7" s="148"/>
+      <c r="F7" s="142"/>
+      <c r="G7" s="148"/>
+      <c r="H7" s="148"/>
+      <c r="I7" s="148"/>
+      <c r="J7" s="148"/>
+      <c r="K7" s="142"/>
       <c r="L7" s="54"/>
       <c r="M7" s="54"/>
       <c r="N7" s="54"/>
@@ -2993,8 +2999,8 @@
       <c r="L8" s="50"/>
       <c r="M8" s="50"/>
       <c r="N8" s="50"/>
-      <c r="O8" s="154"/>
-      <c r="P8" s="155"/>
+      <c r="O8" s="81"/>
+      <c r="P8" s="82"/>
     </row>
     <row r="9" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A9" s="78"/>
@@ -3011,8 +3017,8 @@
       <c r="L9" s="50"/>
       <c r="M9" s="50"/>
       <c r="N9" s="50"/>
-      <c r="O9" s="156"/>
-      <c r="P9" s="155"/>
+      <c r="O9" s="83"/>
+      <c r="P9" s="82"/>
     </row>
     <row r="10" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A10" s="78"/>
@@ -3029,8 +3035,8 @@
       <c r="L10" s="50"/>
       <c r="M10" s="50"/>
       <c r="N10" s="50"/>
-      <c r="O10" s="156"/>
-      <c r="P10" s="155"/>
+      <c r="O10" s="83"/>
+      <c r="P10" s="82"/>
     </row>
     <row r="11" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A11" s="78"/>
@@ -3047,8 +3053,8 @@
       <c r="L11" s="50"/>
       <c r="M11" s="50"/>
       <c r="N11" s="50"/>
-      <c r="O11" s="156"/>
-      <c r="P11" s="155"/>
+      <c r="O11" s="83"/>
+      <c r="P11" s="82"/>
     </row>
     <row r="12" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A12" s="78"/>
@@ -3065,8 +3071,8 @@
       <c r="L12" s="50"/>
       <c r="M12" s="50"/>
       <c r="N12" s="50"/>
-      <c r="O12" s="156"/>
-      <c r="P12" s="155"/>
+      <c r="O12" s="83"/>
+      <c r="P12" s="82"/>
     </row>
     <row r="13" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A13" s="78"/>
@@ -3083,8 +3089,8 @@
       <c r="L13" s="50"/>
       <c r="M13" s="50"/>
       <c r="N13" s="50"/>
-      <c r="O13" s="154"/>
-      <c r="P13" s="155"/>
+      <c r="O13" s="81"/>
+      <c r="P13" s="82"/>
     </row>
     <row r="14" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A14" s="78"/>
@@ -3101,8 +3107,8 @@
       <c r="L14" s="50"/>
       <c r="M14" s="50"/>
       <c r="N14" s="50"/>
-      <c r="O14" s="156"/>
-      <c r="P14" s="155"/>
+      <c r="O14" s="83"/>
+      <c r="P14" s="82"/>
     </row>
     <row r="15" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A15" s="78"/>
@@ -3119,8 +3125,8 @@
       <c r="L15" s="50"/>
       <c r="M15" s="50"/>
       <c r="N15" s="50"/>
-      <c r="O15" s="156"/>
-      <c r="P15" s="155"/>
+      <c r="O15" s="83"/>
+      <c r="P15" s="82"/>
     </row>
     <row r="16" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A16" s="78"/>
@@ -3137,8 +3143,8 @@
       <c r="L16" s="50"/>
       <c r="M16" s="50"/>
       <c r="N16" s="50"/>
-      <c r="O16" s="156"/>
-      <c r="P16" s="155"/>
+      <c r="O16" s="83"/>
+      <c r="P16" s="82"/>
     </row>
     <row r="17" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A17" s="78"/>
@@ -3155,8 +3161,8 @@
       <c r="L17" s="50"/>
       <c r="M17" s="50"/>
       <c r="N17" s="50"/>
-      <c r="O17" s="156"/>
-      <c r="P17" s="155"/>
+      <c r="O17" s="83"/>
+      <c r="P17" s="82"/>
     </row>
     <row r="18" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A18" s="78"/>
@@ -3173,8 +3179,8 @@
       <c r="L18" s="50"/>
       <c r="M18" s="50"/>
       <c r="N18" s="50"/>
-      <c r="O18" s="156"/>
-      <c r="P18" s="155"/>
+      <c r="O18" s="83"/>
+      <c r="P18" s="82"/>
     </row>
     <row r="19" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A19" s="78"/>
@@ -3191,8 +3197,8 @@
       <c r="L19" s="50"/>
       <c r="M19" s="50"/>
       <c r="N19" s="50"/>
-      <c r="O19" s="154"/>
-      <c r="P19" s="155"/>
+      <c r="O19" s="81"/>
+      <c r="P19" s="82"/>
     </row>
     <row r="20" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A20" s="78"/>
@@ -3209,8 +3215,8 @@
       <c r="L20" s="50"/>
       <c r="M20" s="50"/>
       <c r="N20" s="50"/>
-      <c r="O20" s="156"/>
-      <c r="P20" s="155"/>
+      <c r="O20" s="83"/>
+      <c r="P20" s="82"/>
     </row>
     <row r="21" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A21" s="78"/>
@@ -3227,8 +3233,8 @@
       <c r="L21" s="50"/>
       <c r="M21" s="50"/>
       <c r="N21" s="50"/>
-      <c r="O21" s="156"/>
-      <c r="P21" s="155"/>
+      <c r="O21" s="83"/>
+      <c r="P21" s="82"/>
     </row>
     <row r="22" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A22" s="78"/>
@@ -3245,8 +3251,8 @@
       <c r="L22" s="50"/>
       <c r="M22" s="50"/>
       <c r="N22" s="50"/>
-      <c r="O22" s="156"/>
-      <c r="P22" s="155"/>
+      <c r="O22" s="83"/>
+      <c r="P22" s="82"/>
     </row>
     <row r="23" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A23" s="78"/>
@@ -3263,8 +3269,8 @@
       <c r="L23" s="50"/>
       <c r="M23" s="50"/>
       <c r="N23" s="50"/>
-      <c r="O23" s="156"/>
-      <c r="P23" s="155"/>
+      <c r="O23" s="83"/>
+      <c r="P23" s="82"/>
     </row>
     <row r="24" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A24" s="60"/>
@@ -3281,8 +3287,8 @@
       <c r="L24" s="50"/>
       <c r="M24" s="50"/>
       <c r="N24" s="50"/>
-      <c r="O24" s="156"/>
-      <c r="P24" s="155"/>
+      <c r="O24" s="83"/>
+      <c r="P24" s="82"/>
     </row>
     <row r="25" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A25" s="60"/>
@@ -3299,8 +3305,8 @@
       <c r="L25" s="50"/>
       <c r="M25" s="50"/>
       <c r="N25" s="50"/>
-      <c r="O25" s="156"/>
-      <c r="P25" s="155"/>
+      <c r="O25" s="83"/>
+      <c r="P25" s="82"/>
     </row>
     <row r="26" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A26" s="60"/>
@@ -3317,8 +3323,8 @@
       <c r="L26" s="50"/>
       <c r="M26" s="50"/>
       <c r="N26" s="50"/>
-      <c r="O26" s="156"/>
-      <c r="P26" s="155"/>
+      <c r="O26" s="83"/>
+      <c r="P26" s="82"/>
     </row>
     <row r="27" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A27" s="60"/>
@@ -3335,8 +3341,8 @@
       <c r="L27" s="50"/>
       <c r="M27" s="50"/>
       <c r="N27" s="50"/>
-      <c r="O27" s="156"/>
-      <c r="P27" s="155"/>
+      <c r="O27" s="83"/>
+      <c r="P27" s="82"/>
       <c r="Q27" s="48"/>
       <c r="R27" s="48"/>
     </row>
@@ -3370,8 +3376,8 @@
         <f>SUM(N8:N27)</f>
         <v>0</v>
       </c>
-      <c r="O28" s="157"/>
-      <c r="P28" s="158"/>
+      <c r="O28" s="84"/>
+      <c r="P28" s="85"/>
       <c r="Q28" s="47"/>
       <c r="R28" s="48"/>
     </row>
@@ -3379,31 +3385,31 @@
       <c r="A29" s="62" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="139">
+      <c r="B29" s="126">
         <f>B30+F30</f>
         <v>0</v>
       </c>
-      <c r="C29" s="140"/>
-      <c r="D29" s="141"/>
+      <c r="C29" s="127"/>
+      <c r="D29" s="128"/>
       <c r="E29" s="46" t="s">
         <v>30</v>
       </c>
       <c r="F29" s="46"/>
       <c r="G29" s="46"/>
-      <c r="H29" s="125" t="s">
+      <c r="H29" s="112" t="s">
         <v>33</v>
       </c>
-      <c r="I29" s="126"/>
-      <c r="J29" s="127"/>
-      <c r="K29" s="145">
+      <c r="I29" s="113"/>
+      <c r="J29" s="114"/>
+      <c r="K29" s="132">
         <f>B31</f>
         <v>0</v>
       </c>
-      <c r="L29" s="146"/>
-      <c r="M29" s="146"/>
-      <c r="N29" s="146"/>
-      <c r="O29" s="146"/>
-      <c r="P29" s="147"/>
+      <c r="L29" s="133"/>
+      <c r="M29" s="133"/>
+      <c r="N29" s="133"/>
+      <c r="O29" s="133"/>
+      <c r="P29" s="134"/>
       <c r="Q29" s="47"/>
       <c r="R29" s="48"/>
     </row>
@@ -3411,29 +3417,29 @@
       <c r="A30" s="62" t="s">
         <v>40</v>
       </c>
-      <c r="B30" s="142">
+      <c r="B30" s="129">
         <f>L28</f>
         <v>0</v>
       </c>
-      <c r="C30" s="143"/>
-      <c r="D30" s="144"/>
+      <c r="C30" s="130"/>
+      <c r="D30" s="131"/>
       <c r="E30" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="F30" s="142">
+      <c r="F30" s="129">
         <f>M28+N28</f>
         <v>0</v>
       </c>
-      <c r="G30" s="144"/>
-      <c r="H30" s="128"/>
-      <c r="I30" s="129"/>
-      <c r="J30" s="130"/>
-      <c r="K30" s="148"/>
-      <c r="L30" s="149"/>
-      <c r="M30" s="149"/>
-      <c r="N30" s="149"/>
-      <c r="O30" s="149"/>
-      <c r="P30" s="150"/>
+      <c r="G30" s="131"/>
+      <c r="H30" s="115"/>
+      <c r="I30" s="116"/>
+      <c r="J30" s="117"/>
+      <c r="K30" s="135"/>
+      <c r="L30" s="136"/>
+      <c r="M30" s="136"/>
+      <c r="N30" s="136"/>
+      <c r="O30" s="136"/>
+      <c r="P30" s="137"/>
       <c r="Q30" s="47"/>
       <c r="R30" s="48"/>
     </row>
@@ -3441,29 +3447,29 @@
       <c r="A31" s="62" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="134">
+      <c r="B31" s="121">
         <f>K28</f>
         <v>0</v>
       </c>
-      <c r="C31" s="135"/>
-      <c r="D31" s="136"/>
+      <c r="C31" s="122"/>
+      <c r="D31" s="123"/>
       <c r="E31" s="56" t="s">
         <v>36</v>
       </c>
-      <c r="F31" s="123">
+      <c r="F31" s="110">
         <f>D28</f>
         <v>0</v>
       </c>
-      <c r="G31" s="124"/>
-      <c r="H31" s="128"/>
-      <c r="I31" s="129"/>
-      <c r="J31" s="130"/>
-      <c r="K31" s="148"/>
-      <c r="L31" s="149"/>
-      <c r="M31" s="149"/>
-      <c r="N31" s="149"/>
-      <c r="O31" s="149"/>
-      <c r="P31" s="150"/>
+      <c r="G31" s="111"/>
+      <c r="H31" s="115"/>
+      <c r="I31" s="116"/>
+      <c r="J31" s="117"/>
+      <c r="K31" s="135"/>
+      <c r="L31" s="136"/>
+      <c r="M31" s="136"/>
+      <c r="N31" s="136"/>
+      <c r="O31" s="136"/>
+      <c r="P31" s="137"/>
       <c r="Q31" s="47"/>
       <c r="R31" s="48"/>
     </row>
@@ -3472,41 +3478,29 @@
         <v>38</v>
       </c>
       <c r="B32" s="64"/>
-      <c r="C32" s="137">
+      <c r="C32" s="124">
         <v>0</v>
       </c>
-      <c r="D32" s="138"/>
+      <c r="D32" s="125"/>
       <c r="E32" s="64" t="s">
         <v>39</v>
       </c>
       <c r="F32" s="64"/>
       <c r="G32" s="64"/>
-      <c r="H32" s="131"/>
-      <c r="I32" s="132"/>
-      <c r="J32" s="133"/>
-      <c r="K32" s="151"/>
-      <c r="L32" s="152"/>
-      <c r="M32" s="152"/>
-      <c r="N32" s="152"/>
-      <c r="O32" s="152"/>
-      <c r="P32" s="153"/>
+      <c r="H32" s="118"/>
+      <c r="I32" s="119"/>
+      <c r="J32" s="120"/>
+      <c r="K32" s="138"/>
+      <c r="L32" s="139"/>
+      <c r="M32" s="139"/>
+      <c r="N32" s="139"/>
+      <c r="O32" s="139"/>
+      <c r="P32" s="140"/>
       <c r="Q32" s="48"/>
       <c r="R32" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="H29:J32"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="K29:P32"/>
-    <mergeCell ref="D5:D7"/>
-    <mergeCell ref="E3:I3"/>
     <mergeCell ref="Q5:R5"/>
     <mergeCell ref="J3:K3"/>
     <mergeCell ref="A4:C4"/>
@@ -3523,6 +3517,18 @@
     <mergeCell ref="K5:K7"/>
     <mergeCell ref="J5:J7"/>
     <mergeCell ref="E5:E7"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="H29:J32"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="K29:P32"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="E3:I3"/>
   </mergeCells>
   <phoneticPr fontId="27" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update the xlsx output template
</commit_message>
<xml_diff>
--- a/resources/Out_format.xlsx
+++ b/resources/Out_format.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\my_github\FlightCheckPy\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\Gordon\FlightCheckPy\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA91118-C100-420E-A6EF-FED0183EAF9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA56938-DA8F-466C-A4CD-1D6907438B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="20676" windowHeight="22416" activeTab="1" xr2:uid="{D6DB75D4-A8CC-4A73-9AF5-6E324AED1BA5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{D6DB75D4-A8CC-4A73-9AF5-6E324AED1BA5}"/>
   </bookViews>
   <sheets>
     <sheet name="RECEIPT" sheetId="17" r:id="rId1"/>
@@ -29,8 +29,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -472,14 +470,14 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="8">
-    <numFmt numFmtId="44" formatCode="_ &quot;¥&quot;* #,##0.00_ ;_ &quot;¥&quot;* \-#,##0.00_ ;_ &quot;¥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="26" formatCode="\$#,##0.00_);[Red]\(\$#,##0.00\)"/>
-    <numFmt numFmtId="176" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="178" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="179" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
-    <numFmt numFmtId="180" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="181" formatCode="00000"/>
+    <numFmt numFmtId="176" formatCode="_ &quot;¥&quot;* #,##0.00_ ;_ &quot;¥&quot;* \-#,##0.00_ ;_ &quot;¥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="178" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
+    <numFmt numFmtId="179" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="180" formatCode="00000"/>
   </numFmts>
   <fonts count="44" x14ac:knownFonts="1">
     <font>
@@ -1145,7 +1143,7 @@
   </borders>
   <cellStyleXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="38" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="38" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
@@ -1166,32 +1164,32 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="178" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="177" fontId="12" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="12" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="12" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="12" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1251,7 +1249,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="180" fontId="9" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="179" fontId="9" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="26" fontId="28" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1278,7 +1276,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="180" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="179" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="26" fontId="39" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1301,10 +1299,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="11" xfId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
@@ -1314,7 +1312,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="181" fontId="9" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="180" fontId="9" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1325,217 +1323,11 @@
     <xf numFmtId="0" fontId="41" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="177" fontId="9" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="9" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="9" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="9" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="distributed"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="26" fontId="3" fillId="0" borderId="10" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="10" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1559,78 +1351,284 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="distributed"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="8" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="8" fontId="22" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="177" fontId="22" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="44" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="28" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="28" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="28" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="28" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="28" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="28" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="28" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="8" fontId="28" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="10" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="10" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="10" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="10" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="26" fontId="3" fillId="0" borderId="10" xfId="8" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="176" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="22" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="22" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="178" fontId="22" fillId="0" borderId="3" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="14">
@@ -1895,9 +1893,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1935,9 +1933,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1970,9 +1968,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -2005,9 +2020,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2183,18 +2215,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D40067CD-9956-401A-A618-7A92843119E5}">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:L47"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.44140625" style="1" customWidth="1"/>
-    <col min="3" max="5" width="9.109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.109375" style="1" customWidth="1"/>
-    <col min="7" max="8" width="9.109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="10.88671875" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="1" width="11.625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.5" style="1" customWidth="1"/>
+    <col min="3" max="5" width="9.125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.125" style="1" customWidth="1"/>
+    <col min="7" max="8" width="9.125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="10.875" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2207,37 +2239,37 @@
       <c r="J1" s="3"/>
       <c r="K1" s="3"/>
     </row>
-    <row r="2" spans="1:12" ht="22.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="C2" s="3"/>
-      <c r="D2" s="83" t="s">
+      <c r="D2" s="110" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="83"/>
-      <c r="F2" s="83"/>
+      <c r="E2" s="110"/>
+      <c r="F2" s="110"/>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="25"/>
     </row>
-    <row r="3" spans="1:12" ht="19.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="19.5" x14ac:dyDescent="0.25">
       <c r="A3" s="32"/>
       <c r="B3" s="32"/>
       <c r="C3" s="32"/>
-      <c r="D3" s="84" t="s">
+      <c r="D3" s="111" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="84"/>
-      <c r="F3" s="84"/>
-      <c r="G3" s="85" t="s">
+      <c r="E3" s="111"/>
+      <c r="F3" s="111"/>
+      <c r="G3" s="112" t="s">
         <v>44</v>
       </c>
-      <c r="H3" s="85"/>
-      <c r="I3" s="85"/>
+      <c r="H3" s="112"/>
+      <c r="I3" s="112"/>
       <c r="J3" s="35"/>
       <c r="K3" s="35"/>
       <c r="L3" s="34"/>
     </row>
-    <row r="4" spans="1:12" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" s="24"/>
       <c r="B4" s="24"/>
       <c r="C4" s="24"/>
@@ -2250,203 +2282,203 @@
       <c r="J4" s="24"/>
       <c r="K4" s="24"/>
     </row>
-    <row r="5" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="86" t="s">
+    <row r="5" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="100" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="86"/>
-      <c r="C5" s="87">
+      <c r="B5" s="100"/>
+      <c r="C5" s="118">
         <f>SUM!C13</f>
         <v>0</v>
       </c>
-      <c r="D5" s="87"/>
-      <c r="E5" s="87"/>
-      <c r="F5" s="89" t="s">
+      <c r="D5" s="118"/>
+      <c r="E5" s="118"/>
+      <c r="F5" s="125" t="s">
         <v>46</v>
       </c>
-      <c r="G5" s="185">
+      <c r="G5" s="127">
         <f>SUM!G11</f>
         <v>0</v>
       </c>
-      <c r="H5" s="185"/>
-      <c r="I5" s="185"/>
+      <c r="H5" s="127"/>
+      <c r="I5" s="127"/>
       <c r="J5" s="33"/>
       <c r="K5" s="33"/>
     </row>
-    <row r="6" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="91" t="s">
+    <row r="6" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="120" t="s">
         <v>47</v>
       </c>
-      <c r="B6" s="91"/>
-      <c r="C6" s="88"/>
-      <c r="D6" s="88"/>
-      <c r="E6" s="88"/>
-      <c r="F6" s="90"/>
-      <c r="G6" s="186"/>
-      <c r="H6" s="186"/>
-      <c r="I6" s="186"/>
+      <c r="B6" s="120"/>
+      <c r="C6" s="98"/>
+      <c r="D6" s="98"/>
+      <c r="E6" s="98"/>
+      <c r="F6" s="126"/>
+      <c r="G6" s="128"/>
+      <c r="H6" s="128"/>
+      <c r="I6" s="128"/>
       <c r="J6" s="33"/>
       <c r="K6" s="33"/>
     </row>
-    <row r="8" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="92" t="s">
+    <row r="8" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="122" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="92"/>
-      <c r="C8" s="93" t="s">
+      <c r="B8" s="122"/>
+      <c r="C8" s="123" t="s">
         <v>79</v>
       </c>
-      <c r="D8" s="93"/>
-      <c r="E8" s="93"/>
-      <c r="F8" s="93"/>
-      <c r="G8" s="93"/>
-      <c r="H8" s="93"/>
-      <c r="I8" s="93"/>
-    </row>
-    <row r="9" spans="1:12" ht="49.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="92"/>
-      <c r="B9" s="92"/>
-      <c r="C9" s="94"/>
-      <c r="D9" s="94"/>
-      <c r="E9" s="94"/>
-      <c r="F9" s="94"/>
-      <c r="G9" s="94"/>
-      <c r="H9" s="94"/>
-      <c r="I9" s="94"/>
-    </row>
-    <row r="11" spans="1:12" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A11" s="86" t="s">
+      <c r="D8" s="123"/>
+      <c r="E8" s="123"/>
+      <c r="F8" s="123"/>
+      <c r="G8" s="123"/>
+      <c r="H8" s="123"/>
+      <c r="I8" s="123"/>
+    </row>
+    <row r="9" spans="1:12" ht="49.7" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="122"/>
+      <c r="B9" s="122"/>
+      <c r="C9" s="124"/>
+      <c r="D9" s="124"/>
+      <c r="E9" s="124"/>
+      <c r="F9" s="124"/>
+      <c r="G9" s="124"/>
+      <c r="H9" s="124"/>
+      <c r="I9" s="124"/>
+    </row>
+    <row r="11" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A11" s="100" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="86"/>
-      <c r="C11" s="87" t="s">
+      <c r="B11" s="100"/>
+      <c r="C11" s="118" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="87"/>
-      <c r="E11" s="87"/>
+      <c r="D11" s="118"/>
+      <c r="E11" s="118"/>
       <c r="F11" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="G11" s="95">
+      <c r="G11" s="119">
         <f>SUM!C14</f>
         <v>0</v>
       </c>
-      <c r="H11" s="87"/>
-      <c r="I11" s="87"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="91" t="s">
+      <c r="H11" s="118"/>
+      <c r="I11" s="118"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12" s="120" t="s">
         <v>50</v>
       </c>
-      <c r="B12" s="91"/>
-      <c r="C12" s="88"/>
-      <c r="D12" s="88"/>
-      <c r="E12" s="88"/>
+      <c r="B12" s="120"/>
+      <c r="C12" s="98"/>
+      <c r="D12" s="98"/>
+      <c r="E12" s="98"/>
       <c r="F12" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="88"/>
-      <c r="H12" s="88"/>
-      <c r="I12" s="88"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="86" t="s">
+      <c r="G12" s="98"/>
+      <c r="H12" s="98"/>
+      <c r="I12" s="98"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" s="100" t="s">
         <v>52</v>
       </c>
-      <c r="B14" s="86"/>
-      <c r="C14" s="87" t="s">
+      <c r="B14" s="100"/>
+      <c r="C14" s="118" t="s">
         <v>76</v>
       </c>
-      <c r="D14" s="87"/>
-      <c r="E14" s="87"/>
-      <c r="F14" s="87"/>
-      <c r="G14" s="87"/>
-      <c r="H14" s="87"/>
-      <c r="I14" s="87"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="91" t="s">
+      <c r="D14" s="118"/>
+      <c r="E14" s="118"/>
+      <c r="F14" s="118"/>
+      <c r="G14" s="118"/>
+      <c r="H14" s="118"/>
+      <c r="I14" s="118"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A15" s="120" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="91"/>
-      <c r="C15" s="88"/>
-      <c r="D15" s="88"/>
-      <c r="E15" s="88"/>
-      <c r="F15" s="88"/>
-      <c r="G15" s="88"/>
-      <c r="H15" s="88"/>
-      <c r="I15" s="88"/>
-    </row>
-    <row r="17" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="120"/>
+      <c r="C15" s="98"/>
+      <c r="D15" s="98"/>
+      <c r="E15" s="98"/>
+      <c r="F15" s="98"/>
+      <c r="G15" s="98"/>
+      <c r="H15" s="98"/>
+      <c r="I15" s="98"/>
+    </row>
+    <row r="17" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="B17" s="87" t="s">
+      <c r="B17" s="118" t="s">
         <v>55</v>
       </c>
-      <c r="C17" s="87"/>
-      <c r="D17" s="87"/>
-      <c r="E17" s="87"/>
+      <c r="C17" s="118"/>
+      <c r="D17" s="118"/>
+      <c r="E17" s="118"/>
       <c r="F17" s="31" t="s">
         <v>56</v>
       </c>
       <c r="G17" s="31"/>
-      <c r="H17" s="87" t="s">
+      <c r="H17" s="118" t="s">
         <v>57</v>
       </c>
-      <c r="I17" s="87"/>
-    </row>
-    <row r="18" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I17" s="118"/>
+    </row>
+    <row r="18" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="B18" s="88"/>
-      <c r="C18" s="88"/>
-      <c r="D18" s="88"/>
-      <c r="E18" s="88"/>
-      <c r="F18" s="96" t="s">
+      <c r="B18" s="98"/>
+      <c r="C18" s="98"/>
+      <c r="D18" s="98"/>
+      <c r="E18" s="98"/>
+      <c r="F18" s="121" t="s">
         <v>59</v>
       </c>
-      <c r="G18" s="97"/>
-      <c r="H18" s="88"/>
-      <c r="I18" s="88"/>
-    </row>
-    <row r="20" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G18" s="103"/>
+      <c r="H18" s="98"/>
+      <c r="I18" s="98"/>
+    </row>
+    <row r="20" spans="1:9" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="B20" s="87" t="s">
+      <c r="B20" s="118" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="87"/>
-      <c r="D20" s="87"/>
-      <c r="E20" s="87"/>
+      <c r="C20" s="118"/>
+      <c r="D20" s="118"/>
+      <c r="E20" s="118"/>
       <c r="F20" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="G20" s="95">
+      <c r="G20" s="119">
         <f>SUM!C14</f>
         <v>0</v>
       </c>
-      <c r="H20" s="87"/>
-      <c r="I20" s="87"/>
-    </row>
-    <row r="21" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H20" s="118"/>
+      <c r="I20" s="118"/>
+    </row>
+    <row r="21" spans="1:9" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="27" t="s">
         <v>62</v>
       </c>
-      <c r="B21" s="88"/>
-      <c r="C21" s="88"/>
-      <c r="D21" s="88"/>
-      <c r="E21" s="88"/>
+      <c r="B21" s="98"/>
+      <c r="C21" s="98"/>
+      <c r="D21" s="98"/>
+      <c r="E21" s="98"/>
       <c r="F21" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="G21" s="88"/>
-      <c r="H21" s="88"/>
-      <c r="I21" s="88"/>
-    </row>
-    <row r="22" spans="1:9" ht="19.8" x14ac:dyDescent="0.35">
+      <c r="G21" s="98"/>
+      <c r="H21" s="98"/>
+      <c r="I21" s="98"/>
+    </row>
+    <row r="22" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
       <c r="A22" s="27"/>
       <c r="B22" s="28"/>
       <c r="C22" s="28"/>
@@ -2457,43 +2489,43 @@
       <c r="H22" s="28"/>
       <c r="I22" s="28"/>
     </row>
-    <row r="23" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="166" t="s">
+    <row r="23" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A24" s="108" t="s">
         <v>86</v>
       </c>
-      <c r="B24" s="167"/>
-      <c r="C24" s="167"/>
-      <c r="D24" s="167"/>
-      <c r="E24" s="167"/>
-      <c r="F24" s="167"/>
-      <c r="G24" s="167"/>
-      <c r="H24" s="167"/>
-      <c r="I24" s="167"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="168"/>
-      <c r="B25" s="169"/>
-      <c r="C25" s="169"/>
-      <c r="D25" s="169"/>
-      <c r="E25" s="169"/>
-      <c r="F25" s="169"/>
-      <c r="G25" s="169"/>
-      <c r="H25" s="169"/>
-      <c r="I25" s="169"/>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="168"/>
-      <c r="B26" s="169"/>
-      <c r="C26" s="169"/>
-      <c r="D26" s="169"/>
-      <c r="E26" s="169"/>
-      <c r="F26" s="169"/>
-      <c r="G26" s="169"/>
-      <c r="H26" s="169"/>
-      <c r="I26" s="169"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B24" s="109"/>
+      <c r="C24" s="109"/>
+      <c r="D24" s="109"/>
+      <c r="E24" s="109"/>
+      <c r="F24" s="109"/>
+      <c r="G24" s="109"/>
+      <c r="H24" s="109"/>
+      <c r="I24" s="109"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A25" s="93"/>
+      <c r="B25" s="94"/>
+      <c r="C25" s="94"/>
+      <c r="D25" s="94"/>
+      <c r="E25" s="94"/>
+      <c r="F25" s="94"/>
+      <c r="G25" s="94"/>
+      <c r="H25" s="94"/>
+      <c r="I25" s="94"/>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A26" s="93"/>
+      <c r="B26" s="94"/>
+      <c r="C26" s="94"/>
+      <c r="D26" s="94"/>
+      <c r="E26" s="94"/>
+      <c r="F26" s="94"/>
+      <c r="G26" s="94"/>
+      <c r="H26" s="94"/>
+      <c r="I26" s="94"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -2504,34 +2536,34 @@
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
     </row>
-    <row r="28" spans="1:9" ht="22.2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="C28" s="3"/>
-      <c r="D28" s="83" t="s">
+      <c r="D28" s="110" t="s">
         <v>42</v>
       </c>
-      <c r="E28" s="83"/>
-      <c r="F28" s="83"/>
+      <c r="E28" s="110"/>
+      <c r="F28" s="110"/>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
       <c r="I28" s="25"/>
     </row>
-    <row r="29" spans="1:9" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A29" s="170"/>
-      <c r="B29" s="170"/>
-      <c r="C29" s="170"/>
-      <c r="D29" s="84" t="s">
+    <row r="29" spans="1:9" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="95"/>
+      <c r="B29" s="95"/>
+      <c r="C29" s="95"/>
+      <c r="D29" s="111" t="s">
         <v>43</v>
       </c>
-      <c r="E29" s="84"/>
-      <c r="F29" s="84"/>
-      <c r="G29" s="85" t="s">
+      <c r="E29" s="111"/>
+      <c r="F29" s="111"/>
+      <c r="G29" s="112" t="s">
         <v>44</v>
       </c>
-      <c r="H29" s="85"/>
-      <c r="I29" s="85"/>
-    </row>
-    <row r="30" spans="1:9" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="H29" s="112"/>
+      <c r="I29" s="112"/>
+    </row>
+    <row r="30" spans="1:9" ht="18" x14ac:dyDescent="0.25">
       <c r="A30" s="24"/>
       <c r="B30" s="24"/>
       <c r="C30" s="24"/>
@@ -2542,215 +2574,223 @@
       <c r="H30" s="24"/>
       <c r="I30" s="24"/>
     </row>
-    <row r="31" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="86" t="s">
+    <row r="31" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="100" t="s">
         <v>45</v>
       </c>
-      <c r="B31" s="86"/>
-      <c r="C31" s="171">
+      <c r="B31" s="100"/>
+      <c r="C31" s="97">
         <f>C5</f>
         <v>0</v>
       </c>
-      <c r="D31" s="171"/>
-      <c r="E31" s="171"/>
-      <c r="F31" s="172" t="s">
+      <c r="D31" s="97"/>
+      <c r="E31" s="97"/>
+      <c r="F31" s="113" t="s">
         <v>46</v>
       </c>
-      <c r="G31" s="173">
+      <c r="G31" s="115">
         <f>G5</f>
         <v>0</v>
       </c>
-      <c r="H31" s="174"/>
-      <c r="I31" s="174"/>
-    </row>
-    <row r="32" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="175" t="s">
+      <c r="H31" s="116"/>
+      <c r="I31" s="116"/>
+    </row>
+    <row r="32" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="101" t="s">
         <v>47</v>
       </c>
-      <c r="B32" s="175"/>
-      <c r="C32" s="88"/>
-      <c r="D32" s="88"/>
-      <c r="E32" s="88"/>
-      <c r="F32" s="176"/>
-      <c r="G32" s="177"/>
-      <c r="H32" s="177"/>
-      <c r="I32" s="177"/>
-    </row>
-    <row r="34" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="178" t="s">
+      <c r="B32" s="101"/>
+      <c r="C32" s="98"/>
+      <c r="D32" s="98"/>
+      <c r="E32" s="98"/>
+      <c r="F32" s="114"/>
+      <c r="G32" s="117"/>
+      <c r="H32" s="117"/>
+      <c r="I32" s="117"/>
+    </row>
+    <row r="34" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="104" t="s">
         <v>20</v>
       </c>
-      <c r="B34" s="179"/>
-      <c r="C34" s="180" t="str">
+      <c r="B34" s="105"/>
+      <c r="C34" s="106" t="str">
         <f>C8</f>
         <v>No Cash</v>
       </c>
-      <c r="D34" s="180"/>
-      <c r="E34" s="180"/>
-      <c r="F34" s="180"/>
-      <c r="G34" s="180"/>
-      <c r="H34" s="180"/>
-      <c r="I34" s="180"/>
-    </row>
-    <row r="35" spans="1:9" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="179"/>
-      <c r="B35" s="179"/>
-      <c r="C35" s="181"/>
-      <c r="D35" s="181"/>
-      <c r="E35" s="181"/>
-      <c r="F35" s="181"/>
-      <c r="G35" s="181"/>
-      <c r="H35" s="181"/>
-      <c r="I35" s="181"/>
-    </row>
-    <row r="37" spans="1:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="86" t="s">
+      <c r="D34" s="106"/>
+      <c r="E34" s="106"/>
+      <c r="F34" s="106"/>
+      <c r="G34" s="106"/>
+      <c r="H34" s="106"/>
+      <c r="I34" s="106"/>
+    </row>
+    <row r="35" spans="1:9" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="105"/>
+      <c r="B35" s="105"/>
+      <c r="C35" s="107"/>
+      <c r="D35" s="107"/>
+      <c r="E35" s="107"/>
+      <c r="F35" s="107"/>
+      <c r="G35" s="107"/>
+      <c r="H35" s="107"/>
+      <c r="I35" s="107"/>
+    </row>
+    <row r="37" spans="1:9" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="100" t="s">
         <v>19</v>
       </c>
-      <c r="B37" s="86"/>
-      <c r="C37" s="171" t="s">
+      <c r="B37" s="100"/>
+      <c r="C37" s="97" t="s">
         <v>48</v>
       </c>
-      <c r="D37" s="171"/>
-      <c r="E37" s="171"/>
+      <c r="D37" s="97"/>
+      <c r="E37" s="97"/>
       <c r="F37" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="G37" s="182">
+      <c r="G37" s="99">
         <f>G11</f>
         <v>0</v>
       </c>
-      <c r="H37" s="171"/>
-      <c r="I37" s="171"/>
-    </row>
-    <row r="38" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="175" t="s">
+      <c r="H37" s="97"/>
+      <c r="I37" s="97"/>
+    </row>
+    <row r="38" spans="1:9" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="101" t="s">
         <v>50</v>
       </c>
-      <c r="B38" s="175"/>
-      <c r="C38" s="88"/>
-      <c r="D38" s="88"/>
-      <c r="E38" s="88"/>
-      <c r="F38" s="183" t="s">
+      <c r="B38" s="101"/>
+      <c r="C38" s="98"/>
+      <c r="D38" s="98"/>
+      <c r="E38" s="98"/>
+      <c r="F38" s="96" t="s">
         <v>51</v>
       </c>
-      <c r="G38" s="88"/>
-      <c r="H38" s="88"/>
-      <c r="I38" s="88"/>
-    </row>
-    <row r="40" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="86" t="s">
+      <c r="G38" s="98"/>
+      <c r="H38" s="98"/>
+      <c r="I38" s="98"/>
+    </row>
+    <row r="40" spans="1:9" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="100" t="s">
         <v>52</v>
       </c>
-      <c r="B40" s="86"/>
-      <c r="C40" s="171" t="s">
+      <c r="B40" s="100"/>
+      <c r="C40" s="97" t="s">
         <v>87</v>
       </c>
-      <c r="D40" s="171"/>
-      <c r="E40" s="171"/>
-      <c r="F40" s="171"/>
-      <c r="G40" s="171"/>
-      <c r="H40" s="171"/>
-      <c r="I40" s="171"/>
-    </row>
-    <row r="41" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="175" t="s">
+      <c r="D40" s="97"/>
+      <c r="E40" s="97"/>
+      <c r="F40" s="97"/>
+      <c r="G40" s="97"/>
+      <c r="H40" s="97"/>
+      <c r="I40" s="97"/>
+    </row>
+    <row r="41" spans="1:9" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="101" t="s">
         <v>53</v>
       </c>
-      <c r="B41" s="175"/>
-      <c r="C41" s="88"/>
-      <c r="D41" s="88"/>
-      <c r="E41" s="88"/>
-      <c r="F41" s="88"/>
-      <c r="G41" s="88"/>
-      <c r="H41" s="88"/>
-      <c r="I41" s="88"/>
-    </row>
-    <row r="43" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="101"/>
+      <c r="C41" s="98"/>
+      <c r="D41" s="98"/>
+      <c r="E41" s="98"/>
+      <c r="F41" s="98"/>
+      <c r="G41" s="98"/>
+      <c r="H41" s="98"/>
+      <c r="I41" s="98"/>
+    </row>
+    <row r="43" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="B43" s="171" t="s">
+      <c r="B43" s="97" t="s">
         <v>55</v>
       </c>
-      <c r="C43" s="171"/>
-      <c r="D43" s="171"/>
-      <c r="E43" s="171"/>
+      <c r="C43" s="97"/>
+      <c r="D43" s="97"/>
+      <c r="E43" s="97"/>
       <c r="F43" s="30" t="s">
         <v>56</v>
       </c>
       <c r="G43" s="30"/>
-      <c r="H43" s="171" t="s">
+      <c r="H43" s="97" t="s">
         <v>57</v>
       </c>
-      <c r="I43" s="171"/>
-    </row>
-    <row r="44" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I43" s="97"/>
+    </row>
+    <row r="44" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B44" s="88"/>
-      <c r="C44" s="88"/>
-      <c r="D44" s="88"/>
-      <c r="E44" s="88"/>
-      <c r="F44" s="184" t="s">
+      <c r="B44" s="98"/>
+      <c r="C44" s="98"/>
+      <c r="D44" s="98"/>
+      <c r="E44" s="98"/>
+      <c r="F44" s="102" t="s">
         <v>59</v>
       </c>
-      <c r="G44" s="97"/>
-      <c r="H44" s="88"/>
-      <c r="I44" s="88"/>
-    </row>
-    <row r="46" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G44" s="103"/>
+      <c r="H44" s="98"/>
+      <c r="I44" s="98"/>
+    </row>
+    <row r="46" spans="1:9" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="B46" s="171" t="s">
+      <c r="B46" s="97" t="s">
         <v>55</v>
       </c>
-      <c r="C46" s="171"/>
-      <c r="D46" s="171"/>
-      <c r="E46" s="171"/>
+      <c r="C46" s="97"/>
+      <c r="D46" s="97"/>
+      <c r="E46" s="97"/>
       <c r="F46" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="G46" s="182">
+      <c r="G46" s="99">
         <f>G20</f>
         <v>0</v>
       </c>
-      <c r="H46" s="171"/>
-      <c r="I46" s="171"/>
-    </row>
-    <row r="47" spans="1:9" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H46" s="97"/>
+      <c r="I46" s="97"/>
+    </row>
+    <row r="47" spans="1:9" ht="13.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B47" s="88"/>
-      <c r="C47" s="88"/>
-      <c r="D47" s="88"/>
-      <c r="E47" s="88"/>
-      <c r="F47" s="183" t="s">
+      <c r="B47" s="98"/>
+      <c r="C47" s="98"/>
+      <c r="D47" s="98"/>
+      <c r="E47" s="98"/>
+      <c r="F47" s="96" t="s">
         <v>63</v>
       </c>
-      <c r="G47" s="88"/>
-      <c r="H47" s="88"/>
-      <c r="I47" s="88"/>
+      <c r="G47" s="98"/>
+      <c r="H47" s="98"/>
+      <c r="I47" s="98"/>
     </row>
   </sheetData>
   <mergeCells count="45">
-    <mergeCell ref="B46:E47"/>
-    <mergeCell ref="G46:I47"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="C40:I41"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="B43:E44"/>
-    <mergeCell ref="H43:I44"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="A34:B35"/>
-    <mergeCell ref="C34:I35"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="C37:E38"/>
-    <mergeCell ref="G37:I38"/>
-    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="G5:I6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A8:B9"/>
+    <mergeCell ref="C8:I9"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:E12"/>
+    <mergeCell ref="G11:I12"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="B20:E21"/>
+    <mergeCell ref="G20:I21"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:I15"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="B17:E18"/>
+    <mergeCell ref="H17:I18"/>
+    <mergeCell ref="F18:G18"/>
     <mergeCell ref="A24:I24"/>
     <mergeCell ref="D28:F28"/>
     <mergeCell ref="D29:F29"/>
@@ -2760,28 +2800,20 @@
     <mergeCell ref="F31:F32"/>
     <mergeCell ref="G31:I32"/>
     <mergeCell ref="A32:B32"/>
-    <mergeCell ref="B20:E21"/>
-    <mergeCell ref="G20:I21"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:I15"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="B17:E18"/>
-    <mergeCell ref="H17:I18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="A8:B9"/>
-    <mergeCell ref="C8:I9"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:E12"/>
-    <mergeCell ref="G11:I12"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="G5:I6"/>
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A34:B35"/>
+    <mergeCell ref="C34:I35"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="C37:E38"/>
+    <mergeCell ref="G37:I38"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="B46:E47"/>
+    <mergeCell ref="G46:I47"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="C40:I41"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="B43:E44"/>
+    <mergeCell ref="H43:I44"/>
+    <mergeCell ref="F44:G44"/>
   </mergeCells>
   <phoneticPr fontId="40" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2798,26 +2830,26 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N26"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.88671875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16.109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.44140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="3.375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5" style="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.6640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="15.44140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="16.44140625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="16.109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="11.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.44140625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="10.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="9.109375" style="1"/>
+    <col min="7" max="7" width="15.625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.5" style="1" customWidth="1"/>
+    <col min="10" max="10" width="16.625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="16.125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5" style="1" customWidth="1"/>
+    <col min="14" max="14" width="10.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="15" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2830,7 +2862,7 @@
       <c r="J1" s="36"/>
       <c r="K1" s="37"/>
     </row>
-    <row r="2" spans="1:14" ht="19.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="19.5" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -2842,25 +2874,25 @@
       <c r="J2" s="3"/>
       <c r="K2" s="25"/>
     </row>
-    <row r="3" spans="1:14" ht="19.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="101" t="s">
+    <row r="3" spans="1:14" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="132" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="101"/>
-      <c r="C3" s="101"/>
-      <c r="D3" s="101"/>
-      <c r="E3" s="101"/>
-      <c r="F3" s="101"/>
-      <c r="G3" s="101"/>
-      <c r="H3" s="101"/>
-      <c r="I3" s="101"/>
-      <c r="J3" s="101"/>
-      <c r="K3" s="101"/>
+      <c r="B3" s="132"/>
+      <c r="C3" s="132"/>
+      <c r="D3" s="132"/>
+      <c r="E3" s="132"/>
+      <c r="F3" s="132"/>
+      <c r="G3" s="132"/>
+      <c r="H3" s="132"/>
+      <c r="I3" s="132"/>
+      <c r="J3" s="132"/>
+      <c r="K3" s="132"/>
       <c r="L3" s="23"/>
       <c r="M3" s="23"/>
       <c r="N3" s="23"/>
     </row>
-    <row r="4" spans="1:14" ht="22.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A4" s="24"/>
       <c r="B4" s="24"/>
       <c r="C4" s="24"/>
@@ -2880,7 +2912,7 @@
       <c r="M4" s="23"/>
       <c r="N4" s="23"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -2893,7 +2925,7 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:14" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="22" t="s">
         <v>18</v>
       </c>
@@ -2910,59 +2942,59 @@
         <v>00-Jan-1900</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="21"/>
-      <c r="B7" s="104" t="s">
+      <c r="B7" s="135" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="98" t="s">
+      <c r="C7" s="129" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="98" t="s">
+      <c r="D7" s="129" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="98" t="s">
+      <c r="E7" s="129" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="98" t="s">
+      <c r="F7" s="129" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="98" t="s">
+      <c r="G7" s="129" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="102" t="s">
+      <c r="H7" s="133" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="103"/>
-      <c r="J7" s="98" t="s">
+      <c r="I7" s="134"/>
+      <c r="J7" s="129" t="s">
         <v>10</v>
       </c>
-      <c r="K7" s="98" t="s">
+      <c r="K7" s="129" t="s">
         <v>9</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="8"/>
     </row>
-    <row r="8" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="21"/>
-      <c r="B8" s="104"/>
-      <c r="C8" s="98"/>
-      <c r="D8" s="98"/>
-      <c r="E8" s="98"/>
-      <c r="F8" s="98"/>
-      <c r="G8" s="98"/>
+      <c r="B8" s="135"/>
+      <c r="C8" s="129"/>
+      <c r="D8" s="129"/>
+      <c r="E8" s="129"/>
+      <c r="F8" s="129"/>
+      <c r="G8" s="129"/>
       <c r="H8" s="20" t="s">
         <v>8</v>
       </c>
       <c r="I8" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="J8" s="98"/>
-      <c r="K8" s="98"/>
+      <c r="J8" s="129"/>
+      <c r="K8" s="129"/>
       <c r="L8" s="2"/>
       <c r="M8" s="8"/>
     </row>
-    <row r="9" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="13">
         <v>1</v>
       </c>
@@ -3002,7 +3034,7 @@
       <c r="L9" s="2"/>
       <c r="M9" s="15"/>
     </row>
-    <row r="10" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="13">
         <v>2</v>
       </c>
@@ -3020,7 +3052,7 @@
       <c r="M10" s="15"/>
       <c r="N10" s="8"/>
     </row>
-    <row r="11" spans="1:14" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="13">
         <v>6</v>
       </c>
@@ -3063,7 +3095,7 @@
       <c r="L11" s="2"/>
       <c r="M11" s="8"/>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="D12" s="3"/>
@@ -3075,7 +3107,7 @@
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>6</v>
       </c>
@@ -3094,7 +3126,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>4</v>
       </c>
@@ -3116,7 +3148,7 @@
         <v>00-Jan-1900</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="6"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -3129,7 +3161,7 @@
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="D16" s="3"/>
@@ -3141,7 +3173,7 @@
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -3154,7 +3186,7 @@
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -3167,7 +3199,7 @@
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="5"/>
@@ -3180,7 +3212,7 @@
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="5"/>
@@ -3193,27 +3225,27 @@
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
     </row>
-    <row r="21" spans="1:11" ht="15" x14ac:dyDescent="0.25">
-      <c r="C21" s="99"/>
-      <c r="D21" s="100"/>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="15" x14ac:dyDescent="0.2">
+      <c r="C21" s="130"/>
+      <c r="D21" s="131"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
     </row>
@@ -3248,92 +3280,92 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" customWidth="1"/>
-    <col min="3" max="3" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" customWidth="1"/>
-    <col min="6" max="6" width="7.6640625" customWidth="1"/>
-    <col min="7" max="7" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.44140625" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="18.5" customWidth="1"/>
+    <col min="2" max="2" width="16.125" customWidth="1"/>
+    <col min="3" max="3" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5" customWidth="1"/>
+    <col min="5" max="5" width="13.625" customWidth="1"/>
+    <col min="6" max="6" width="7.625" customWidth="1"/>
+    <col min="7" max="7" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5" customWidth="1"/>
+    <col min="9" max="9" width="11.625" customWidth="1"/>
     <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="11" max="11" width="10.6640625" customWidth="1"/>
-    <col min="12" max="12" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.109375" customWidth="1"/>
+    <col min="11" max="11" width="10.625" customWidth="1"/>
+    <col min="12" max="12" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.125" customWidth="1"/>
     <col min="14" max="14" width="11" customWidth="1"/>
-    <col min="15" max="15" width="14.44140625" customWidth="1"/>
-    <col min="16" max="16" width="9.44140625" customWidth="1"/>
-    <col min="17" max="17" width="13.6640625" customWidth="1"/>
-    <col min="18" max="18" width="12.33203125" customWidth="1"/>
+    <col min="15" max="15" width="14.5" customWidth="1"/>
+    <col min="16" max="16" width="9.5" customWidth="1"/>
+    <col min="17" max="17" width="13.625" customWidth="1"/>
+    <col min="18" max="18" width="12.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="121" t="s">
+    <row r="1" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="142" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="121"/>
-      <c r="C1" s="121"/>
-      <c r="D1" s="121"/>
-      <c r="E1" s="121"/>
-      <c r="F1" s="121"/>
-      <c r="G1" s="121"/>
-      <c r="H1" s="121"/>
-      <c r="I1" s="121"/>
-      <c r="J1" s="121"/>
-      <c r="K1" s="121"/>
-      <c r="L1" s="121"/>
-      <c r="M1" s="121"/>
-      <c r="N1" s="121"/>
-      <c r="O1" s="121"/>
-      <c r="P1" s="121"/>
+      <c r="B1" s="142"/>
+      <c r="C1" s="142"/>
+      <c r="D1" s="142"/>
+      <c r="E1" s="142"/>
+      <c r="F1" s="142"/>
+      <c r="G1" s="142"/>
+      <c r="H1" s="142"/>
+      <c r="I1" s="142"/>
+      <c r="J1" s="142"/>
+      <c r="K1" s="142"/>
+      <c r="L1" s="142"/>
+      <c r="M1" s="142"/>
+      <c r="N1" s="142"/>
+      <c r="O1" s="142"/>
+      <c r="P1" s="142"/>
       <c r="Q1" s="65"/>
       <c r="R1" s="65"/>
       <c r="S1" s="65"/>
     </row>
-    <row r="2" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="122" t="s">
+    <row r="2" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="143" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="122"/>
-      <c r="C2" s="122"/>
-      <c r="D2" s="122"/>
-      <c r="E2" s="122"/>
-      <c r="F2" s="122"/>
-      <c r="G2" s="122"/>
-      <c r="H2" s="122"/>
-      <c r="I2" s="122"/>
-      <c r="J2" s="122"/>
-      <c r="K2" s="122"/>
-      <c r="L2" s="122"/>
-      <c r="M2" s="122"/>
-      <c r="N2" s="122"/>
-      <c r="O2" s="122"/>
-      <c r="P2" s="122"/>
+      <c r="B2" s="143"/>
+      <c r="C2" s="143"/>
+      <c r="D2" s="143"/>
+      <c r="E2" s="143"/>
+      <c r="F2" s="143"/>
+      <c r="G2" s="143"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="143"/>
+      <c r="J2" s="143"/>
+      <c r="K2" s="143"/>
+      <c r="L2" s="143"/>
+      <c r="M2" s="143"/>
+      <c r="N2" s="143"/>
+      <c r="O2" s="143"/>
+      <c r="P2" s="143"/>
       <c r="Q2" s="66"/>
       <c r="R2" s="66"/>
       <c r="S2" s="66"/>
     </row>
-    <row r="3" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="44" t="s">
         <v>75</v>
       </c>
       <c r="B3" s="44"/>
       <c r="C3" s="44"/>
-      <c r="E3" s="106" t="str">
+      <c r="E3" s="168" t="str">
         <f>"报告期间：" &amp; N3 &amp; "至" &amp; N3</f>
         <v>报告期间：1900年1月0日至1900年1月0日</v>
       </c>
-      <c r="F3" s="106"/>
-      <c r="G3" s="106"/>
-      <c r="H3" s="106"/>
-      <c r="I3" s="106"/>
-      <c r="J3" s="106" t="s">
+      <c r="F3" s="168"/>
+      <c r="G3" s="168"/>
+      <c r="H3" s="168"/>
+      <c r="I3" s="168"/>
+      <c r="J3" s="168" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="106"/>
+      <c r="K3" s="168"/>
       <c r="L3" s="43"/>
       <c r="M3" s="63"/>
       <c r="N3" s="63" t="str">
@@ -3346,18 +3378,18 @@
       <c r="R3" s="50"/>
       <c r="S3" s="45"/>
     </row>
-    <row r="4" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="107" t="s">
+    <row r="4" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="175" t="s">
         <v>73</v>
       </c>
-      <c r="B4" s="107"/>
-      <c r="C4" s="107"/>
+      <c r="B4" s="175"/>
+      <c r="C4" s="175"/>
       <c r="D4" s="67"/>
       <c r="E4" s="67"/>
       <c r="F4" s="68"/>
       <c r="G4" s="69"/>
-      <c r="H4" s="108"/>
-      <c r="I4" s="108"/>
+      <c r="H4" s="176"/>
+      <c r="I4" s="176"/>
       <c r="J4" s="64" t="s">
         <v>74</v>
       </c>
@@ -3371,69 +3403,69 @@
       <c r="O4" s="64"/>
       <c r="P4" s="64"/>
     </row>
-    <row r="5" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="119" t="s">
+    <row r="5" spans="1:19" s="41" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="185" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="117" t="s">
+      <c r="B5" s="183" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="115" t="s">
+      <c r="C5" s="181" t="s">
         <v>70</v>
       </c>
-      <c r="D5" s="111" t="s">
+      <c r="D5" s="166" t="s">
         <v>71</v>
       </c>
-      <c r="E5" s="109" t="s">
+      <c r="E5" s="177" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="111" t="s">
+      <c r="F5" s="166" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="109" t="s">
+      <c r="G5" s="177" t="s">
         <v>26</v>
       </c>
-      <c r="H5" s="109" t="s">
+      <c r="H5" s="177" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="109" t="s">
+      <c r="I5" s="177" t="s">
         <v>28</v>
       </c>
-      <c r="J5" s="109" t="s">
+      <c r="J5" s="177" t="s">
         <v>29</v>
       </c>
-      <c r="K5" s="111" t="s">
+      <c r="K5" s="166" t="s">
         <v>24</v>
       </c>
-      <c r="L5" s="113" t="s">
+      <c r="L5" s="179" t="s">
         <v>39</v>
       </c>
-      <c r="M5" s="113" t="s">
+      <c r="M5" s="179" t="s">
         <v>40</v>
       </c>
-      <c r="N5" s="113"/>
+      <c r="N5" s="179"/>
       <c r="O5" s="55" t="s">
         <v>64</v>
       </c>
       <c r="P5" s="56" t="s">
         <v>65</v>
       </c>
-      <c r="Q5" s="105"/>
-      <c r="R5" s="105"/>
-    </row>
-    <row r="6" spans="1:19" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="120"/>
-      <c r="B6" s="118"/>
-      <c r="C6" s="116"/>
-      <c r="D6" s="112"/>
-      <c r="E6" s="110"/>
-      <c r="F6" s="112"/>
-      <c r="G6" s="110"/>
-      <c r="H6" s="110"/>
-      <c r="I6" s="110"/>
-      <c r="J6" s="110"/>
-      <c r="K6" s="112"/>
-      <c r="L6" s="114"/>
+      <c r="Q5" s="174"/>
+      <c r="R5" s="174"/>
+    </row>
+    <row r="6" spans="1:19" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="186"/>
+      <c r="B6" s="184"/>
+      <c r="C6" s="182"/>
+      <c r="D6" s="167"/>
+      <c r="E6" s="178"/>
+      <c r="F6" s="167"/>
+      <c r="G6" s="178"/>
+      <c r="H6" s="178"/>
+      <c r="I6" s="178"/>
+      <c r="J6" s="178"/>
+      <c r="K6" s="167"/>
+      <c r="L6" s="180"/>
       <c r="M6" s="52" t="s">
         <v>41</v>
       </c>
@@ -3447,18 +3479,18 @@
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A7" s="120"/>
-      <c r="B7" s="118"/>
-      <c r="C7" s="116"/>
-      <c r="D7" s="112"/>
-      <c r="E7" s="110"/>
-      <c r="F7" s="112"/>
-      <c r="G7" s="110"/>
-      <c r="H7" s="110"/>
-      <c r="I7" s="110"/>
-      <c r="J7" s="110"/>
-      <c r="K7" s="112"/>
+    <row r="7" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A7" s="186"/>
+      <c r="B7" s="184"/>
+      <c r="C7" s="182"/>
+      <c r="D7" s="167"/>
+      <c r="E7" s="178"/>
+      <c r="F7" s="167"/>
+      <c r="G7" s="178"/>
+      <c r="H7" s="178"/>
+      <c r="I7" s="178"/>
+      <c r="J7" s="178"/>
+      <c r="K7" s="167"/>
       <c r="L7" s="53"/>
       <c r="M7" s="53"/>
       <c r="N7" s="53"/>
@@ -3469,7 +3501,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A8" s="75"/>
       <c r="B8" s="76"/>
       <c r="C8" s="42"/>
@@ -3487,7 +3519,7 @@
       <c r="O8" s="78"/>
       <c r="P8" s="79"/>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A9" s="75"/>
       <c r="B9" s="77"/>
       <c r="C9" s="42"/>
@@ -3505,7 +3537,7 @@
       <c r="O9" s="80"/>
       <c r="P9" s="79"/>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A10" s="75"/>
       <c r="B10" s="77"/>
       <c r="C10" s="42"/>
@@ -3523,7 +3555,7 @@
       <c r="O10" s="80"/>
       <c r="P10" s="79"/>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A11" s="75"/>
       <c r="B11" s="77"/>
       <c r="C11" s="42"/>
@@ -3541,7 +3573,7 @@
       <c r="O11" s="80"/>
       <c r="P11" s="79"/>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A12" s="75"/>
       <c r="B12" s="77"/>
       <c r="C12" s="42"/>
@@ -3559,7 +3591,7 @@
       <c r="O12" s="80"/>
       <c r="P12" s="79"/>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A13" s="75"/>
       <c r="B13" s="76"/>
       <c r="C13" s="42"/>
@@ -3577,7 +3609,7 @@
       <c r="O13" s="78"/>
       <c r="P13" s="79"/>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A14" s="75"/>
       <c r="B14" s="77"/>
       <c r="C14" s="42"/>
@@ -3595,7 +3627,7 @@
       <c r="O14" s="80"/>
       <c r="P14" s="79"/>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A15" s="75"/>
       <c r="B15" s="77"/>
       <c r="C15" s="42"/>
@@ -3613,7 +3645,7 @@
       <c r="O15" s="80"/>
       <c r="P15" s="79"/>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A16" s="75"/>
       <c r="B16" s="77"/>
       <c r="C16" s="42"/>
@@ -3631,7 +3663,7 @@
       <c r="O16" s="80"/>
       <c r="P16" s="79"/>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A17" s="75"/>
       <c r="B17" s="77"/>
       <c r="C17" s="42"/>
@@ -3649,7 +3681,7 @@
       <c r="O17" s="80"/>
       <c r="P17" s="79"/>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A18" s="75"/>
       <c r="B18" s="77"/>
       <c r="C18" s="42"/>
@@ -3667,7 +3699,7 @@
       <c r="O18" s="80"/>
       <c r="P18" s="79"/>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A19" s="75"/>
       <c r="B19" s="77"/>
       <c r="C19" s="42"/>
@@ -3685,7 +3717,7 @@
       <c r="O19" s="78"/>
       <c r="P19" s="79"/>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A20" s="75"/>
       <c r="B20" s="77"/>
       <c r="C20" s="42"/>
@@ -3703,7 +3735,7 @@
       <c r="O20" s="80"/>
       <c r="P20" s="79"/>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A21" s="75"/>
       <c r="B21" s="77"/>
       <c r="C21" s="42"/>
@@ -3721,7 +3753,7 @@
       <c r="O21" s="80"/>
       <c r="P21" s="79"/>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A22" s="75"/>
       <c r="B22" s="77"/>
       <c r="C22" s="42"/>
@@ -3739,7 +3771,7 @@
       <c r="O22" s="80"/>
       <c r="P22" s="79"/>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A23" s="75"/>
       <c r="B23" s="77"/>
       <c r="C23" s="42"/>
@@ -3757,7 +3789,7 @@
       <c r="O23" s="80"/>
       <c r="P23" s="79"/>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A24" s="58"/>
       <c r="B24" s="48"/>
       <c r="C24" s="42"/>
@@ -3775,7 +3807,7 @@
       <c r="O24" s="80"/>
       <c r="P24" s="79"/>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A25" s="58"/>
       <c r="B25" s="48"/>
       <c r="C25" s="42"/>
@@ -3793,7 +3825,7 @@
       <c r="O25" s="80"/>
       <c r="P25" s="79"/>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A26" s="58"/>
       <c r="B26" s="48"/>
       <c r="C26" s="42"/>
@@ -3811,7 +3843,7 @@
       <c r="O26" s="80"/>
       <c r="P26" s="79"/>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A27" s="58"/>
       <c r="B27" s="48"/>
       <c r="C27" s="42"/>
@@ -3831,31 +3863,31 @@
       <c r="Q27" s="47"/>
       <c r="R27" s="47"/>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A28" s="152" t="s">
+    <row r="28" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A28" s="83" t="s">
         <v>80</v>
       </c>
-      <c r="B28" s="153"/>
-      <c r="C28" s="152" t="s">
+      <c r="B28" s="84"/>
+      <c r="C28" s="83" t="s">
         <v>81</v>
       </c>
-      <c r="D28" s="154">
-        <f>COUNT(D8:D27D2:D27)</f>
+      <c r="D28" s="85">
+        <f>COUNT(D8:D27)</f>
         <v>0</v>
       </c>
-      <c r="E28" s="155"/>
-      <c r="F28" s="156"/>
-      <c r="G28" s="157" t="s">
+      <c r="E28" s="86"/>
+      <c r="F28" s="87"/>
+      <c r="G28" s="88" t="s">
         <v>82</v>
       </c>
-      <c r="H28" s="158">
+      <c r="H28" s="89">
         <f>COUNTIF(H8:H27,"*Seat*")</f>
         <v>0</v>
       </c>
-      <c r="I28" s="157" t="s">
+      <c r="I28" s="88" t="s">
         <v>85</v>
       </c>
-      <c r="J28" s="159">
+      <c r="J28" s="90">
         <f>COUNTIF(H8:H27,"*EXPC*")</f>
         <v>0</v>
       </c>
@@ -3880,39 +3912,39 @@
       <c r="Q28" s="46"/>
       <c r="R28" s="47"/>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A29" s="59" t="s">
         <v>34</v>
       </c>
-      <c r="B29" s="138">
+      <c r="B29" s="169">
         <f>B30+F30</f>
         <v>0</v>
       </c>
-      <c r="C29" s="139"/>
-      <c r="D29" s="160" t="s">
+      <c r="C29" s="170"/>
+      <c r="D29" s="91" t="s">
         <v>30</v>
       </c>
-      <c r="E29" s="161"/>
+      <c r="E29" s="92"/>
       <c r="F29" s="140"/>
-      <c r="G29" s="142"/>
-      <c r="H29" s="125" t="s">
+      <c r="G29" s="141"/>
+      <c r="H29" s="146" t="s">
         <v>33</v>
       </c>
-      <c r="I29" s="126"/>
-      <c r="J29" s="127"/>
-      <c r="K29" s="143">
+      <c r="I29" s="147"/>
+      <c r="J29" s="148"/>
+      <c r="K29" s="157">
         <f>B31</f>
         <v>0</v>
       </c>
-      <c r="L29" s="144"/>
-      <c r="M29" s="144"/>
-      <c r="N29" s="144"/>
-      <c r="O29" s="144"/>
-      <c r="P29" s="145"/>
+      <c r="L29" s="158"/>
+      <c r="M29" s="158"/>
+      <c r="N29" s="158"/>
+      <c r="O29" s="158"/>
+      <c r="P29" s="159"/>
       <c r="Q29" s="46"/>
       <c r="R29" s="47"/>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A30" s="59" t="s">
         <v>38</v>
       </c>
@@ -3920,101 +3952,86 @@
         <f>L28</f>
         <v>0</v>
       </c>
-      <c r="C30" s="141"/>
-      <c r="D30" s="164" t="s">
+      <c r="C30" s="171"/>
+      <c r="D30" s="136" t="s">
         <v>83</v>
       </c>
-      <c r="E30" s="165"/>
+      <c r="E30" s="137"/>
       <c r="F30" s="140">
         <f>M28+N28</f>
         <v>0</v>
       </c>
-      <c r="G30" s="142"/>
-      <c r="H30" s="128"/>
-      <c r="I30" s="129"/>
-      <c r="J30" s="130"/>
-      <c r="K30" s="146"/>
-      <c r="L30" s="147"/>
-      <c r="M30" s="147"/>
-      <c r="N30" s="147"/>
-      <c r="O30" s="147"/>
-      <c r="P30" s="148"/>
+      <c r="G30" s="141"/>
+      <c r="H30" s="149"/>
+      <c r="I30" s="150"/>
+      <c r="J30" s="151"/>
+      <c r="K30" s="160"/>
+      <c r="L30" s="161"/>
+      <c r="M30" s="161"/>
+      <c r="N30" s="161"/>
+      <c r="O30" s="161"/>
+      <c r="P30" s="162"/>
       <c r="Q30" s="46"/>
       <c r="R30" s="47"/>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A31" s="59" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="134">
+      <c r="B31" s="172">
         <f>K28</f>
         <v>0</v>
       </c>
-      <c r="C31" s="135"/>
-      <c r="D31" s="162" t="s">
+      <c r="C31" s="173"/>
+      <c r="D31" s="138" t="s">
         <v>84</v>
       </c>
-      <c r="E31" s="163"/>
-      <c r="F31" s="123">
+      <c r="E31" s="139"/>
+      <c r="F31" s="144">
         <f>D28</f>
         <v>0</v>
       </c>
-      <c r="G31" s="124"/>
-      <c r="H31" s="128"/>
-      <c r="I31" s="129"/>
-      <c r="J31" s="130"/>
-      <c r="K31" s="146"/>
-      <c r="L31" s="147"/>
-      <c r="M31" s="147"/>
-      <c r="N31" s="147"/>
-      <c r="O31" s="147"/>
-      <c r="P31" s="148"/>
+      <c r="G31" s="145"/>
+      <c r="H31" s="149"/>
+      <c r="I31" s="150"/>
+      <c r="J31" s="151"/>
+      <c r="K31" s="160"/>
+      <c r="L31" s="161"/>
+      <c r="M31" s="161"/>
+      <c r="N31" s="161"/>
+      <c r="O31" s="161"/>
+      <c r="P31" s="162"/>
       <c r="Q31" s="46"/>
       <c r="R31" s="47"/>
     </row>
-    <row r="32" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="60" t="s">
         <v>36</v>
       </c>
       <c r="B32" s="61"/>
-      <c r="C32" s="136">
+      <c r="C32" s="155">
         <v>0</v>
       </c>
-      <c r="D32" s="137"/>
+      <c r="D32" s="156"/>
       <c r="E32" s="61" t="s">
         <v>37</v>
       </c>
       <c r="F32" s="61"/>
       <c r="G32" s="61"/>
-      <c r="H32" s="131"/>
-      <c r="I32" s="132"/>
-      <c r="J32" s="133"/>
-      <c r="K32" s="149"/>
-      <c r="L32" s="150"/>
-      <c r="M32" s="150"/>
-      <c r="N32" s="150"/>
-      <c r="O32" s="150"/>
-      <c r="P32" s="151"/>
+      <c r="H32" s="152"/>
+      <c r="I32" s="153"/>
+      <c r="J32" s="154"/>
+      <c r="K32" s="163"/>
+      <c r="L32" s="164"/>
+      <c r="M32" s="164"/>
+      <c r="N32" s="164"/>
+      <c r="O32" s="164"/>
+      <c r="P32" s="165"/>
       <c r="Q32" s="47"/>
       <c r="R32" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="H29:J32"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="K29:P32"/>
-    <mergeCell ref="D5:D7"/>
-    <mergeCell ref="E3:I3"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
     <mergeCell ref="Q5:R5"/>
     <mergeCell ref="J3:K3"/>
     <mergeCell ref="A4:C4"/>
@@ -4031,10 +4048,25 @@
     <mergeCell ref="K5:K7"/>
     <mergeCell ref="J5:J7"/>
     <mergeCell ref="E5:E7"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="H29:J32"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="K29:P32"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
   </mergeCells>
   <phoneticPr fontId="27" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="71" fitToHeight="0" orientation="landscape" verticalDpi="0" r:id="rId1"/>
+  <pageSetup scale="71" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter>
     <oddHeader xml:space="preserve">&amp;RORIGINAL          COPY     
 </oddHeader>

</xml_diff>